<commit_message>
[看板] D32 完成, 02/03 部署验收 6/6
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-19.xlsx
+++ b/docs/progress/显性目的进度_2026-10-19.xlsx
@@ -8522,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J183"/>
+  <dimension ref="A1:J184"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8593,16 +8593,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.9347826086956522</v>
+        <v>0.9565217391304348</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>43/46</t>
+          <t>44/46</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 24/25 + 交付 19/21 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 24/25 + 交付 20/21 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8625,16 +8625,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.8135593220338984</v>
+        <v>0.8305084745762712</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>48/59</t>
+          <t>49/59</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 16/24 + 交付 32/35 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 16/24 + 交付 33/35 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8657,16 +8657,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.734375</v>
+        <v>0.75</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>47/64</t>
+          <t>48/64</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 14/24 + 交付 33/40 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 14/24 + 交付 34/40 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8778,13 +8778,13 @@
         <v>46314</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.9348</v>
+        <v>0.9565</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0.8136</v>
+        <v>0.8305</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.7344000000000001</v>
+        <v>0.75</v>
       </c>
     </row>
     <row r="12">
@@ -9768,51 +9768,51 @@
     </row>
     <row r="54">
       <c r="A54" s="17" t="n">
-        <v>46313</v>
-      </c>
-      <c r="B54" s="6" t="inlineStr">
-        <is>
-          <t>长跑</t>
+        <v>46314</v>
+      </c>
+      <c r="B54" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D32</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
+          <t>开机画面期间推流立即接上合主线 8bff92e: 根因 bootscr 本机连 voxslice:9500 占到 --hold 60 释放, serve 一次一个客户端; 改为外来客户端接入即断 bootscr; 02/03 卡上 voxslice → 4ac8a7f0 (旧 .bak-d32), 重启验收两块都 6/6, 开机后约 1 min 推流 1351 帧/90 s</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1017_03_24h</t>
+          <t>progress/v0_accept/acc32_*.log</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="17" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B55" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46313</v>
+      </c>
+      <c r="B55" s="6" t="inlineStr">
+        <is>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>D27</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
+          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/SPEC.md</t>
+          <t>progress/soak_v0/1017_03_24h</t>
         </is>
       </c>
     </row>
@@ -9820,24 +9820,24 @@
       <c r="A56" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B56" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B56" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>V2-5</t>
+          <t>D27</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
+          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_fmt/README.md</t>
+          <t>dr1v90 d27_link/SPEC.md</t>
         </is>
       </c>
     </row>
@@ -9852,17 +9852,17 @@
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>D28b</t>
+          <t>V2-5</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
+          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/回板当天.md</t>
+          <t>dr1v90 v2_fmt/README.md</t>
         </is>
       </c>
     </row>
@@ -9870,24 +9870,24 @@
       <c r="A58" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B58" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>进展</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>D27b</t>
+          <t>D28b</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
+          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/README.md</t>
+          <t>dr1v90 v1_bringup/回板当天.md</t>
         </is>
       </c>
     </row>
@@ -9895,24 +9895,24 @@
       <c r="A59" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B59" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B59" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>V2-6</t>
+          <t>D27b</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
+          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 gw5a_bridge/p2/README.md</t>
+          <t>dr1v90 d27_link/README.md</t>
         </is>
       </c>
     </row>
@@ -9922,22 +9922,22 @@
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>全套</t>
+          <t>V2-6</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
+          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ~/full_*.log</t>
+          <t>dr1v90 gw5a_bridge/p2/README.md</t>
         </is>
       </c>
     </row>
@@ -9947,22 +9947,22 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>修复</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>全套</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
+          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 slice/SPEC.md §13.2</t>
+          <t>dr1v90 ~/full_*.log</t>
         </is>
       </c>
     </row>
@@ -9972,22 +9972,22 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
+          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1016_wkend_24h</t>
+          <t>dr1v90 slice/SPEC.md §13.2</t>
         </is>
       </c>
     </row>
@@ -9997,7 +9997,7 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -10007,37 +10007,37 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
+          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1017_*.log</t>
+          <t>progress/soak_v0/1016_wkend_24h</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>部署</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
+          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22c.board.log</t>
+          <t>progress/v0_accept/accept_1017_*.log</t>
         </is>
       </c>
     </row>
@@ -10045,9 +10045,9 @@
       <c r="A65" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B65" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -10057,12 +10057,12 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
+          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d22c.board.log</t>
         </is>
       </c>
     </row>
@@ -10070,24 +10070,24 @@
       <c r="A66" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B66" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B66" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
+          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board5.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10095,9 +10095,9 @@
       <c r="A67" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
@@ -10107,12 +10107,12 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
+          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d21.board5.log</t>
         </is>
       </c>
     </row>
@@ -10127,12 +10127,12 @@
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
+          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
@@ -10145,9 +10145,9 @@
       <c r="A69" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B69" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B69" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
@@ -10157,12 +10157,12 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
+          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_A fps_B</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10170,9 +10170,9 @@
       <c r="A70" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B70" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
@@ -10182,12 +10182,12 @@
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
+          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_C</t>
+          <t>soak_runs/fps_A fps_B</t>
         </is>
       </c>
     </row>
@@ -10195,24 +10195,24 @@
       <c r="A71" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B71" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
+          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20d-ackrps db4ec93</t>
+          <t>soak_runs/fps_C</t>
         </is>
       </c>
     </row>
@@ -10227,17 +10227,17 @@
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
+          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
+          <t>dr1v90 task/d20d-ackrps db4ec93</t>
         </is>
       </c>
     </row>
@@ -10247,22 +10247,22 @@
       </c>
       <c r="B73" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
+          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_D</t>
+          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
         </is>
       </c>
     </row>
@@ -10270,9 +10270,9 @@
       <c r="A74" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B74" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B74" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
@@ -10282,12 +10282,12 @@
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
+          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>soak_runs/fps_D</t>
         </is>
       </c>
     </row>
@@ -10295,24 +10295,24 @@
       <c r="A75" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B75" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
+          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>~/rv_deploy.board.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10320,24 +10320,24 @@
       <c r="A76" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
+          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_deploy.board.log</t>
         </is>
       </c>
     </row>
@@ -10345,24 +10345,24 @@
       <c r="A77" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>验收</t>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
+          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10372,22 +10372,22 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>开工</t>
+          <t>验收</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>D20e/D23</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
+          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
+          <t>progress/v0_accept/</t>
         </is>
       </c>
     </row>
@@ -10395,24 +10395,24 @@
       <c r="A79" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B79" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>开工</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D24</t>
+          <t>D20e/D23</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
+          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>用户</t>
+          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
         </is>
       </c>
     </row>
@@ -10420,24 +10420,24 @@
       <c r="A80" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B80" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B80" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D24</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
+          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
@@ -10452,12 +10452,12 @@
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
+          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
@@ -10470,24 +10470,24 @@
       <c r="A82" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B82" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B82" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
+          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1016_d20e.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10495,24 +10495,24 @@
       <c r="A83" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B83" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>KR7.3/D24</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
+          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/v0_accept/accept_1016_d20e.log</t>
         </is>
       </c>
     </row>
@@ -10520,24 +10520,24 @@
       <c r="A84" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>KR7.3/D24</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
+          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>D:\card03</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10545,24 +10545,24 @@
       <c r="A85" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B85" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>D25</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
+          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>D:\card03</t>
         </is>
       </c>
     </row>
@@ -10570,24 +10570,24 @@
       <c r="A86" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B86" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D25</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
+          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\cap_COM29.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10602,17 +10602,17 @@
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
+          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20d_ackrps d20c_fps</t>
+          <t>D:\card03\cap_COM29.log</t>
         </is>
       </c>
     </row>
@@ -10620,24 +10620,24 @@
       <c r="A88" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B88" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
+          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d12_latency/RESULTS.md</t>
+          <t>dr1v90 d20d_ackrps d20c_fps</t>
         </is>
       </c>
     </row>
@@ -10652,17 +10652,17 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
+          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d9_e2e/</t>
+          <t>dr1v90 d12_latency/RESULTS.md</t>
         </is>
       </c>
     </row>
@@ -10670,24 +10670,24 @@
       <c r="A90" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B90" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B90" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
+          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\boot03.log</t>
+          <t>dr1v90 d9_e2e/</t>
         </is>
       </c>
     </row>
@@ -10695,24 +10695,24 @@
       <c r="A91" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B91" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D26</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
+          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
+          <t>D:\card03\boot03.log</t>
         </is>
       </c>
     </row>
@@ -10720,24 +10720,24 @@
       <c r="A92" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>开工</t>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>周末</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
+          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
+          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
         </is>
       </c>
     </row>
@@ -10747,22 +10747,22 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>方案</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>D29</t>
+          <t>周末</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
+          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d29_sdboot/PLAN.md</t>
+          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
         </is>
       </c>
     </row>
@@ -10770,24 +10770,24 @@
       <c r="A94" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B94" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>方案</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D28</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
+          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/</t>
+          <t>dr1v90 d29_sdboot/PLAN.md</t>
         </is>
       </c>
     </row>
@@ -10795,24 +10795,24 @@
       <c r="A95" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>修复</t>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D30</t>
+          <t>D28</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
+          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
+          <t>dr1v90 v1_bringup/</t>
         </is>
       </c>
     </row>
@@ -10822,22 +10822,22 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>V2-3</t>
+          <t>D30</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
+          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_map/DESIGN.md</t>
+          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
         </is>
       </c>
     </row>
@@ -10847,47 +10847,47 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>评估</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>V2-3</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
+          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d31_v1odd/REPORT.md</t>
+          <t>dr1v90 v2_map/DESIGN.md</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B98" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B98" s="6" t="inlineStr">
+        <is>
+          <t>评估</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>dr1v90 d31_v1odd/REPORT.md</t>
         </is>
       </c>
     </row>
@@ -10895,24 +10895,24 @@
       <c r="A99" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -10927,17 +10927,17 @@
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -10945,24 +10945,24 @@
       <c r="A101" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B101" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -10977,12 +10977,12 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
@@ -10995,24 +10995,24 @@
       <c r="A103" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B103" s="6" t="inlineStr">
-        <is>
-          <t>分析</t>
+      <c r="B103" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11020,24 +11020,24 @@
       <c r="A104" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B104" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B104" s="6" t="inlineStr">
+        <is>
+          <t>分析</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -11045,19 +11045,19 @@
       <c r="A105" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B105" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
@@ -11070,24 +11070,24 @@
       <c r="A106" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -11095,24 +11095,24 @@
       <c r="A107" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B107" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B107" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -11120,24 +11120,24 @@
       <c r="A108" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B108" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -11152,17 +11152,17 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -11172,22 +11172,22 @@
       </c>
       <c r="B110" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -11195,24 +11195,24 @@
       <c r="A111" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B111" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B111" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -11220,24 +11220,24 @@
       <c r="A112" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B112" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11247,22 +11247,22 @@
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -11270,24 +11270,24 @@
       <c r="A114" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B114" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -11295,9 +11295,9 @@
       <c r="A115" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B115" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B115" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
@@ -11307,12 +11307,12 @@
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11327,17 +11327,17 @@
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -11347,7 +11347,7 @@
       </c>
       <c r="B117" s="6" t="inlineStr">
         <is>
-          <t>复验</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
@@ -11357,12 +11357,12 @@
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -11372,22 +11372,22 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>复验</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -11395,9 +11395,9 @@
       <c r="A119" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B119" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
@@ -11407,12 +11407,12 @@
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -11420,24 +11420,24 @@
       <c r="A120" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B120" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B120" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11445,24 +11445,24 @@
       <c r="A121" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B121" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B121" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -11477,17 +11477,17 @@
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -11507,7 +11507,7 @@
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
@@ -11520,9 +11520,9 @@
       <c r="A124" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
@@ -11532,12 +11532,12 @@
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -11547,22 +11547,22 @@
       </c>
       <c r="B125" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
@@ -11577,17 +11577,17 @@
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
@@ -11597,7 +11597,7 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
@@ -11607,12 +11607,12 @@
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
@@ -11622,7 +11622,7 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
@@ -11632,12 +11632,12 @@
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
@@ -11647,47 +11647,47 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B130" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B130" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -11695,24 +11695,24 @@
       <c r="A131" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B131" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -11720,24 +11720,24 @@
       <c r="A132" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B132" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B132" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -11757,7 +11757,7 @@
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
@@ -11770,24 +11770,24 @@
       <c r="A134" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B134" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B134" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11795,24 +11795,24 @@
       <c r="A135" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B135" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B135" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -11820,9 +11820,9 @@
       <c r="A136" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B136" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
@@ -11832,12 +11832,12 @@
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -11845,9 +11845,9 @@
       <c r="A137" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B137" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B137" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
@@ -11857,12 +11857,12 @@
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -11870,24 +11870,24 @@
       <c r="A138" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B138" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11895,24 +11895,24 @@
       <c r="A139" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B139" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B139" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -11920,24 +11920,24 @@
       <c r="A140" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B140" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B140" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -11945,24 +11945,24 @@
       <c r="A141" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B141" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B141" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11970,9 +11970,9 @@
       <c r="A142" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B142" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B142" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
@@ -11982,12 +11982,12 @@
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -11995,24 +11995,24 @@
       <c r="A143" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B143" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B143" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -12020,9 +12020,9 @@
       <c r="A144" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B144" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B144" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
@@ -12032,12 +12032,12 @@
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12045,24 +12045,24 @@
       <c r="A145" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B145" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B145" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -12070,24 +12070,24 @@
       <c r="A146" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B146" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B146" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12095,24 +12095,24 @@
       <c r="A147" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B147" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B147" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -12120,24 +12120,24 @@
       <c r="A148" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B148" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B148" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -12145,24 +12145,24 @@
       <c r="A149" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B149" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B149" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
@@ -12170,24 +12170,24 @@
       <c r="A150" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B150" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B150" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
@@ -12195,49 +12195,49 @@
       <c r="A151" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B151" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B151" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B152" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B152" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -12252,17 +12252,17 @@
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -12277,17 +12277,17 @@
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -12295,9 +12295,9 @@
       <c r="A155" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B155" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B155" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C155" s="7" t="inlineStr">
@@ -12307,12 +12307,12 @@
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -12320,9 +12320,9 @@
       <c r="A156" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B156" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B156" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C156" s="7" t="inlineStr">
@@ -12332,12 +12332,12 @@
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -12345,24 +12345,24 @@
       <c r="A157" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B157" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B157" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -12370,9 +12370,9 @@
       <c r="A158" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B158" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B158" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C158" s="7" t="inlineStr">
@@ -12382,12 +12382,12 @@
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12402,17 +12402,17 @@
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -12420,9 +12420,9 @@
       <c r="A160" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B160" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B160" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C160" s="7" t="inlineStr">
@@ -12432,12 +12432,12 @@
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -12457,7 +12457,7 @@
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
@@ -12470,24 +12470,24 @@
       <c r="A162" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B162" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B162" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12495,24 +12495,24 @@
       <c r="A163" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B163" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B163" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -12520,24 +12520,24 @@
       <c r="A164" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B164" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B164" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E164" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12552,17 +12552,17 @@
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -12570,19 +12570,19 @@
       <c r="A166" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B166" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B166" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C166" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E166" s="7" t="inlineStr">
@@ -12595,9 +12595,9 @@
       <c r="A167" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B167" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B167" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C167" s="7" t="inlineStr">
@@ -12607,12 +12607,12 @@
       </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12620,24 +12620,24 @@
       <c r="A168" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B168" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B168" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C168" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -12645,9 +12645,9 @@
       <c r="A169" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B169" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B169" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C169" s="7" t="inlineStr">
@@ -12657,12 +12657,12 @@
       </c>
       <c r="D169" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12670,9 +12670,9 @@
       <c r="A170" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B170" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B170" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C170" s="7" t="inlineStr">
@@ -12682,12 +12682,12 @@
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -12695,24 +12695,24 @@
       <c r="A171" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B171" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B171" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C171" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D171" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12720,24 +12720,24 @@
       <c r="A172" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B172" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B172" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C172" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -12750,15 +12750,19 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C173" s="7" t="inlineStr"/>
+      <c r="C173" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12766,15 +12770,15 @@
       <c r="A174" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B174" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B174" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C174" s="7" t="inlineStr"/>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E174" s="7" t="inlineStr">
@@ -12787,20 +12791,20 @@
       <c r="A175" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B175" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B175" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C175" s="7" t="inlineStr"/>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12813,19 +12817,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C176" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="C176" s="7" t="inlineStr"/>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E176" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -12840,12 +12840,12 @@
       </c>
       <c r="C177" s="7" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D177" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
@@ -12865,12 +12865,12 @@
       </c>
       <c r="C178" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D178" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E178" s="7" t="inlineStr">
@@ -12890,12 +12890,12 @@
       </c>
       <c r="C179" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D179" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
@@ -12915,12 +12915,12 @@
       </c>
       <c r="C180" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E180" s="7" t="inlineStr">
@@ -12940,17 +12940,17 @@
       </c>
       <c r="C181" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D15;D16</t>
         </is>
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12958,24 +12958,24 @@
       <c r="A182" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B182" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B182" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C182" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>KR5.2</t>
         </is>
       </c>
       <c r="D182" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
         </is>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 49031f6</t>
         </is>
       </c>
     </row>
@@ -12983,18 +12983,43 @@
       <c r="A183" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B183" s="19" t="inlineStr">
+      <c r="B183" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C183" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D183" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E183" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B184" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C183" s="7" t="inlineStr"/>
-      <c r="D183" s="7" t="inlineStr">
+      <c r="C184" s="7" t="inlineStr"/>
+      <c r="D184" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E183" s="7" t="inlineStr">
+      <c r="E184" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -17855,7 +17880,7 @@
         <v>28</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="12">
@@ -19567,15 +19592,17 @@
       <c r="E67" s="17" t="n">
         <v>46316</v>
       </c>
-      <c r="F67" s="17" t="n"/>
-      <c r="G67" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F67" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G67" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H67" s="7" t="inlineStr">
         <is>
-          <t>task/d32-bootpush (agent 进行中)</t>
+          <t>合主线 8bff92e; 开机屏让位外来推流, 开机 30 s 推流首 ACK 0.04 s; 02/03 部署 (voxslice 4ac8a7f0) 重启验收 6/6, 推流 1351 帧/90 s 满速</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[看板] 用户拍板 B1/B2/B3、D29、D27 套; 新开 D33/D34/V2-7
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-19.xlsx
+++ b/docs/progress/显性目的进度_2026-10-19.xlsx
@@ -8522,7 +8522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J184"/>
+  <dimension ref="A1:J185"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8625,16 +8625,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.8305084745762712</v>
+        <v>0.8032786885245902</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>49/59</t>
+          <t>49/61</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 16/24 + 交付 33/35 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 16/24 + 交付 33/37 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8657,16 +8657,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.75</v>
+        <v>0.7313432835820896</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>48/64</t>
+          <t>49/67</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 14/24 + 交付 34/40 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 14/24 + 交付 35/43 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8781,10 +8781,10 @@
         <v>0.9565</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0.8305</v>
+        <v>0.8033</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.75</v>
+        <v>0.7313</v>
       </c>
     </row>
     <row r="12">
@@ -9793,51 +9793,51 @@
     </row>
     <row r="55">
       <c r="A55" s="17" t="n">
-        <v>46313</v>
-      </c>
-      <c r="B55" s="6" t="inlineStr">
-        <is>
-          <t>长跑</t>
+        <v>46314</v>
+      </c>
+      <c r="B55" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>用户</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
+          <t>用户拍板: 批准 D29 (03 uboot.env 已换, 旧版 .bak-d29, 热重启 OK, 等冷上电 20 次); V1 回板用 D27 套; B1 V1 改奇数档 357/285/209; B2 24 Hz 用满档 (357 档上沿 ≥12 rps, 桥余量约 0.7%, 回板实测); B3 V2 档表 605/513/461 → 开 D34; 并开 D33 主控灌桥位流 / V2-7 板端 2 期后端 / V0 差距盘点</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1017_03_24h</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="17" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B56" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46313</v>
+      </c>
+      <c r="B56" s="6" t="inlineStr">
+        <is>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>D27</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
+          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/SPEC.md</t>
+          <t>progress/soak_v0/1017_03_24h</t>
         </is>
       </c>
     </row>
@@ -9845,24 +9845,24 @@
       <c r="A57" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B57" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B57" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>V2-5</t>
+          <t>D27</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
+          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_fmt/README.md</t>
+          <t>dr1v90 d27_link/SPEC.md</t>
         </is>
       </c>
     </row>
@@ -9877,17 +9877,17 @@
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>D28b</t>
+          <t>V2-5</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
+          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/回板当天.md</t>
+          <t>dr1v90 v2_fmt/README.md</t>
         </is>
       </c>
     </row>
@@ -9895,24 +9895,24 @@
       <c r="A59" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B59" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B59" s="6" t="inlineStr">
+        <is>
+          <t>进展</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>D27b</t>
+          <t>D28b</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
+          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/README.md</t>
+          <t>dr1v90 v1_bringup/回板当天.md</t>
         </is>
       </c>
     </row>
@@ -9920,24 +9920,24 @@
       <c r="A60" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B60" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B60" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>V2-6</t>
+          <t>D27b</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
+          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 gw5a_bridge/p2/README.md</t>
+          <t>dr1v90 d27_link/README.md</t>
         </is>
       </c>
     </row>
@@ -9947,22 +9947,22 @@
       </c>
       <c r="B61" s="6" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>全套</t>
+          <t>V2-6</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
+          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ~/full_*.log</t>
+          <t>dr1v90 gw5a_bridge/p2/README.md</t>
         </is>
       </c>
     </row>
@@ -9972,22 +9972,22 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>修复</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>全套</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
+          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 slice/SPEC.md §13.2</t>
+          <t>dr1v90 ~/full_*.log</t>
         </is>
       </c>
     </row>
@@ -9997,22 +9997,22 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
+          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1016_wkend_24h</t>
+          <t>dr1v90 slice/SPEC.md §13.2</t>
         </is>
       </c>
     </row>
@@ -10022,7 +10022,7 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
@@ -10032,37 +10032,37 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
+          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1017_*.log</t>
+          <t>progress/soak_v0/1016_wkend_24h</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>部署</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
+          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22c.board.log</t>
+          <t>progress/v0_accept/accept_1017_*.log</t>
         </is>
       </c>
     </row>
@@ -10070,9 +10070,9 @@
       <c r="A66" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B66" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B66" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
@@ -10082,12 +10082,12 @@
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
+          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d22c.board.log</t>
         </is>
       </c>
     </row>
@@ -10095,24 +10095,24 @@
       <c r="A67" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B67" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B67" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
+          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board5.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10120,9 +10120,9 @@
       <c r="A68" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B68" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
@@ -10132,12 +10132,12 @@
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
+          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d21.board5.log</t>
         </is>
       </c>
     </row>
@@ -10152,12 +10152,12 @@
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
+          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
@@ -10170,9 +10170,9 @@
       <c r="A70" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B70" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B70" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
@@ -10182,12 +10182,12 @@
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
+          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_A fps_B</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10195,9 +10195,9 @@
       <c r="A71" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B71" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
@@ -10207,12 +10207,12 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
+          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_C</t>
+          <t>soak_runs/fps_A fps_B</t>
         </is>
       </c>
     </row>
@@ -10220,24 +10220,24 @@
       <c r="A72" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B72" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B72" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
+          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20d-ackrps db4ec93</t>
+          <t>soak_runs/fps_C</t>
         </is>
       </c>
     </row>
@@ -10252,17 +10252,17 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
+          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
+          <t>dr1v90 task/d20d-ackrps db4ec93</t>
         </is>
       </c>
     </row>
@@ -10272,22 +10272,22 @@
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
+          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_D</t>
+          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
         </is>
       </c>
     </row>
@@ -10295,9 +10295,9 @@
       <c r="A75" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B75" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B75" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -10307,12 +10307,12 @@
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
+          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>soak_runs/fps_D</t>
         </is>
       </c>
     </row>
@@ -10320,24 +10320,24 @@
       <c r="A76" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
+          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>~/rv_deploy.board.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10345,24 +10345,24 @@
       <c r="A77" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B77" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
+          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_deploy.board.log</t>
         </is>
       </c>
     </row>
@@ -10370,24 +10370,24 @@
       <c r="A78" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B78" s="6" t="inlineStr">
-        <is>
-          <t>验收</t>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
+          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10397,22 +10397,22 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>开工</t>
+          <t>验收</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D20e/D23</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
+          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
+          <t>progress/v0_accept/</t>
         </is>
       </c>
     </row>
@@ -10420,24 +10420,24 @@
       <c r="A80" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B80" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B80" s="6" t="inlineStr">
+        <is>
+          <t>开工</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D24</t>
+          <t>D20e/D23</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
+          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>用户</t>
+          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
         </is>
       </c>
     </row>
@@ -10445,24 +10445,24 @@
       <c r="A81" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B81" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B81" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D24</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
+          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
@@ -10477,12 +10477,12 @@
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
+          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
@@ -10495,24 +10495,24 @@
       <c r="A83" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B83" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B83" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
+          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1016_d20e.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10520,24 +10520,24 @@
       <c r="A84" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B84" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>KR7.3/D24</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
+          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/v0_accept/accept_1016_d20e.log</t>
         </is>
       </c>
     </row>
@@ -10545,24 +10545,24 @@
       <c r="A85" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>KR7.3/D24</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
+          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>D:\card03</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10570,24 +10570,24 @@
       <c r="A86" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B86" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B86" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D25</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
+          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>D:\card03</t>
         </is>
       </c>
     </row>
@@ -10595,24 +10595,24 @@
       <c r="A87" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B87" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D25</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
+          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\cap_COM29.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10627,17 +10627,17 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
+          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20d_ackrps d20c_fps</t>
+          <t>D:\card03\cap_COM29.log</t>
         </is>
       </c>
     </row>
@@ -10645,24 +10645,24 @@
       <c r="A89" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B89" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
+          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d12_latency/RESULTS.md</t>
+          <t>dr1v90 d20d_ackrps d20c_fps</t>
         </is>
       </c>
     </row>
@@ -10677,17 +10677,17 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
+          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d9_e2e/</t>
+          <t>dr1v90 d12_latency/RESULTS.md</t>
         </is>
       </c>
     </row>
@@ -10695,24 +10695,24 @@
       <c r="A91" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B91" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B91" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
+          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\boot03.log</t>
+          <t>dr1v90 d9_e2e/</t>
         </is>
       </c>
     </row>
@@ -10720,24 +10720,24 @@
       <c r="A92" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B92" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D26</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
+          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
+          <t>D:\card03\boot03.log</t>
         </is>
       </c>
     </row>
@@ -10745,24 +10745,24 @@
       <c r="A93" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>开工</t>
+      <c r="B93" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>周末</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
+          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
+          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
         </is>
       </c>
     </row>
@@ -10772,22 +10772,22 @@
       </c>
       <c r="B94" s="6" t="inlineStr">
         <is>
-          <t>方案</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D29</t>
+          <t>周末</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
+          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d29_sdboot/PLAN.md</t>
+          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
         </is>
       </c>
     </row>
@@ -10795,24 +10795,24 @@
       <c r="A95" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B95" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B95" s="6" t="inlineStr">
+        <is>
+          <t>方案</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D28</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
+          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/</t>
+          <t>dr1v90 d29_sdboot/PLAN.md</t>
         </is>
       </c>
     </row>
@@ -10820,24 +10820,24 @@
       <c r="A96" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B96" s="6" t="inlineStr">
-        <is>
-          <t>修复</t>
+      <c r="B96" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D30</t>
+          <t>D28</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
+          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
+          <t>dr1v90 v1_bringup/</t>
         </is>
       </c>
     </row>
@@ -10847,22 +10847,22 @@
       </c>
       <c r="B97" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>V2-3</t>
+          <t>D30</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
+          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_map/DESIGN.md</t>
+          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
         </is>
       </c>
     </row>
@@ -10872,47 +10872,47 @@
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>评估</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>V2-3</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
+          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d31_v1odd/REPORT.md</t>
+          <t>dr1v90 v2_map/DESIGN.md</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B99" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B99" s="6" t="inlineStr">
+        <is>
+          <t>评估</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>dr1v90 d31_v1odd/REPORT.md</t>
         </is>
       </c>
     </row>
@@ -10920,24 +10920,24 @@
       <c r="A100" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B100" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -10952,17 +10952,17 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -10970,24 +10970,24 @@
       <c r="A102" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B102" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B102" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -11002,12 +11002,12 @@
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
@@ -11020,24 +11020,24 @@
       <c r="A104" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B104" s="6" t="inlineStr">
-        <is>
-          <t>分析</t>
+      <c r="B104" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11045,24 +11045,24 @@
       <c r="A105" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B105" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B105" s="6" t="inlineStr">
+        <is>
+          <t>分析</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -11070,19 +11070,19 @@
       <c r="A106" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B106" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
@@ -11095,24 +11095,24 @@
       <c r="A107" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B107" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B107" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -11120,24 +11120,24 @@
       <c r="A108" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B108" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -11145,24 +11145,24 @@
       <c r="A109" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B109" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -11177,17 +11177,17 @@
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -11197,22 +11197,22 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -11220,24 +11220,24 @@
       <c r="A112" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B112" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -11245,24 +11245,24 @@
       <c r="A113" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B113" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11272,22 +11272,22 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -11295,24 +11295,24 @@
       <c r="A115" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B115" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B115" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -11320,9 +11320,9 @@
       <c r="A116" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B116" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B116" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
@@ -11332,12 +11332,12 @@
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11352,17 +11352,17 @@
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -11372,7 +11372,7 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>复验</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
@@ -11382,12 +11382,12 @@
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -11397,22 +11397,22 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>复验</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -11420,9 +11420,9 @@
       <c r="A120" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B120" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B120" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
@@ -11432,12 +11432,12 @@
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -11445,24 +11445,24 @@
       <c r="A121" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B121" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B121" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11470,24 +11470,24 @@
       <c r="A122" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B122" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -11502,17 +11502,17 @@
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -11532,7 +11532,7 @@
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
@@ -11545,9 +11545,9 @@
       <c r="A125" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B125" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B125" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
@@ -11557,12 +11557,12 @@
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -11572,22 +11572,22 @@
       </c>
       <c r="B126" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
@@ -11602,17 +11602,17 @@
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
@@ -11622,7 +11622,7 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
@@ -11632,12 +11632,12 @@
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
@@ -11647,7 +11647,7 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
@@ -11657,12 +11657,12 @@
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
@@ -11672,47 +11672,47 @@
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B131" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B131" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -11720,24 +11720,24 @@
       <c r="A132" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B132" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B132" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -11745,24 +11745,24 @@
       <c r="A133" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B133" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B133" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -11782,7 +11782,7 @@
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
@@ -11795,24 +11795,24 @@
       <c r="A135" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B135" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B135" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11820,24 +11820,24 @@
       <c r="A136" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B136" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B136" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -11845,9 +11845,9 @@
       <c r="A137" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B137" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B137" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
@@ -11857,12 +11857,12 @@
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -11870,9 +11870,9 @@
       <c r="A138" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B138" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B138" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
@@ -11882,12 +11882,12 @@
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -11895,24 +11895,24 @@
       <c r="A139" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B139" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B139" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11920,24 +11920,24 @@
       <c r="A140" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B140" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -11945,24 +11945,24 @@
       <c r="A141" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B141" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B141" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -11970,24 +11970,24 @@
       <c r="A142" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B142" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B142" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11995,9 +11995,9 @@
       <c r="A143" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B143" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B143" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
@@ -12007,12 +12007,12 @@
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -12020,24 +12020,24 @@
       <c r="A144" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B144" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B144" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -12045,9 +12045,9 @@
       <c r="A145" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B145" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B145" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
@@ -12057,12 +12057,12 @@
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12070,24 +12070,24 @@
       <c r="A146" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B146" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B146" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -12095,24 +12095,24 @@
       <c r="A147" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B147" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B147" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12120,24 +12120,24 @@
       <c r="A148" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B148" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B148" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -12145,24 +12145,24 @@
       <c r="A149" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B149" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B149" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -12170,24 +12170,24 @@
       <c r="A150" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B150" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B150" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
@@ -12195,24 +12195,24 @@
       <c r="A151" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B151" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B151" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
@@ -12220,49 +12220,49 @@
       <c r="A152" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B152" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B153" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B153" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -12277,17 +12277,17 @@
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -12302,17 +12302,17 @@
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -12320,9 +12320,9 @@
       <c r="A156" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B156" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B156" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C156" s="7" t="inlineStr">
@@ -12332,12 +12332,12 @@
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -12345,9 +12345,9 @@
       <c r="A157" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B157" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B157" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
@@ -12357,12 +12357,12 @@
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -12370,24 +12370,24 @@
       <c r="A158" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B158" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B158" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -12395,9 +12395,9 @@
       <c r="A159" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B159" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B159" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C159" s="7" t="inlineStr">
@@ -12407,12 +12407,12 @@
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12427,17 +12427,17 @@
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -12445,9 +12445,9 @@
       <c r="A161" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B161" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B161" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C161" s="7" t="inlineStr">
@@ -12457,12 +12457,12 @@
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -12482,7 +12482,7 @@
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
@@ -12495,24 +12495,24 @@
       <c r="A163" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B163" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B163" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12520,24 +12520,24 @@
       <c r="A164" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B164" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B164" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E164" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -12545,24 +12545,24 @@
       <c r="A165" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B165" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B165" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12577,17 +12577,17 @@
       </c>
       <c r="C166" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E166" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -12595,19 +12595,19 @@
       <c r="A167" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B167" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B167" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C167" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
@@ -12620,9 +12620,9 @@
       <c r="A168" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B168" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B168" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C168" s="7" t="inlineStr">
@@ -12632,12 +12632,12 @@
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12645,24 +12645,24 @@
       <c r="A169" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B169" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B169" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C169" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D169" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -12670,9 +12670,9 @@
       <c r="A170" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B170" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B170" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C170" s="7" t="inlineStr">
@@ -12682,12 +12682,12 @@
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12695,9 +12695,9 @@
       <c r="A171" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B171" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B171" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C171" s="7" t="inlineStr">
@@ -12707,12 +12707,12 @@
       </c>
       <c r="D171" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -12720,24 +12720,24 @@
       <c r="A172" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B172" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B172" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C172" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12745,24 +12745,24 @@
       <c r="A173" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B173" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B173" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C173" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -12775,15 +12775,19 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C174" s="7" t="inlineStr"/>
+      <c r="C174" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E174" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12791,15 +12795,15 @@
       <c r="A175" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B175" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B175" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C175" s="7" t="inlineStr"/>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
@@ -12812,20 +12816,20 @@
       <c r="A176" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B176" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B176" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C176" s="7" t="inlineStr"/>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E176" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12838,19 +12842,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C177" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="C177" s="7" t="inlineStr"/>
       <c r="D177" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -12865,12 +12865,12 @@
       </c>
       <c r="C178" s="7" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D178" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E178" s="7" t="inlineStr">
@@ -12890,12 +12890,12 @@
       </c>
       <c r="C179" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D179" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
@@ -12915,12 +12915,12 @@
       </c>
       <c r="C180" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E180" s="7" t="inlineStr">
@@ -12940,12 +12940,12 @@
       </c>
       <c r="C181" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
@@ -12965,17 +12965,17 @@
       </c>
       <c r="C182" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D15;D16</t>
         </is>
       </c>
       <c r="D182" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
         </is>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12983,24 +12983,24 @@
       <c r="A183" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B183" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B183" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C183" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>KR5.2</t>
         </is>
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 49031f6</t>
         </is>
       </c>
     </row>
@@ -13008,18 +13008,43 @@
       <c r="A184" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B184" s="19" t="inlineStr">
+      <c r="B184" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C184" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D184" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E184" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B185" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C184" s="7" t="inlineStr"/>
-      <c r="D184" s="7" t="inlineStr">
+      <c r="C185" s="7" t="inlineStr"/>
+      <c r="D185" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E184" s="7" t="inlineStr">
+      <c r="E185" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -17732,7 +17757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H67"/>
+  <dimension ref="A1:H70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17776,7 +17801,7 @@
         <v>46307</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>5</v>
@@ -17790,7 +17815,7 @@
         <v>46308</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>7</v>
@@ -17804,7 +17829,7 @@
         <v>46309</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>8</v>
@@ -17818,7 +17843,7 @@
         <v>46310</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>12</v>
@@ -17832,7 +17857,7 @@
         <v>46311</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>20</v>
@@ -17846,7 +17871,7 @@
         <v>46312</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>28</v>
@@ -17860,7 +17885,7 @@
         <v>46313</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>28</v>
@@ -17874,13 +17899,13 @@
         <v>46314</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C11" s="6" t="n">
         <v>28</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12">
@@ -17888,7 +17913,7 @@
         <v>46315</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C12" s="6" t="n">
         <v>34</v>
@@ -17900,10 +17925,10 @@
         <v>46316</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D13" s="6" t="n"/>
     </row>
@@ -17912,10 +17937,10 @@
         <v>46317</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D14" s="6" t="n"/>
     </row>
@@ -17924,10 +17949,10 @@
         <v>46318</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D15" s="6" t="n"/>
     </row>
@@ -17936,10 +17961,10 @@
         <v>46319</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="D16" s="6" t="n"/>
     </row>
@@ -18954,15 +18979,17 @@
         </is>
       </c>
       <c r="E50" s="17" t="n"/>
-      <c r="F50" s="17" t="n"/>
-      <c r="G50" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F50" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H50" s="7" t="inlineStr">
         <is>
-          <t>10-13 主会话规划</t>
+          <t>用户定档表 605/513/461; 10-13 主会话规划</t>
         </is>
       </c>
     </row>
@@ -19603,6 +19630,114 @@
       <c r="H67" s="7" t="inlineStr">
         <is>
           <t>合主线 8bff92e; 开机屏让位外来推流, 开机 30 s 推流首 ACK 0.04 s; 02/03 部署 (voxslice 4ac8a7f0) 重启验收 6/6, 推流 1351 帧/90 s 满速</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="inlineStr">
+        <is>
+          <t>D33</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>主控经 JTAG 给桥灌位流 (V1 远程升级软件)</t>
+        </is>
+      </c>
+      <c r="C68" s="6" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D68" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E68" s="17" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F68" s="17" t="n"/>
+      <c r="G68" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>task/d33-jtag (agent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>D34</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>V1 奇数档 357/285/209 + 24 Hz 满档 (用户 B1/B2)</t>
+        </is>
+      </c>
+      <c r="C69" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F69" s="17" t="n"/>
+      <c r="G69" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H69" s="7" t="inlineStr">
+        <is>
+          <t>task/d34-v1odd (agent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>V2-7</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>板端 voxslice --disp p2 (2 期后端)</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>2期</t>
+        </is>
+      </c>
+      <c r="E70" s="17" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F70" s="17" t="n"/>
+      <c r="G70" s="15" t="inlineStr">
+        <is>
+          <t>🔄</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>task/v2-disp (agent)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[V0差距] KR4.2 补录 D15b 上板 12-bit 通路实测; V0 达成率 95.7%→97.8%
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-19.xlsx
+++ b/docs/progress/显性目的进度_2026-10-19.xlsx
@@ -15,7 +15,7 @@
     <sheet name="历史记录" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$79</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$80</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -103,12 +103,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00D9D9D9"/>
+        <fgColor rgb="00FFEB9C"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFEB9C"/>
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
     <fill>
@@ -231,10 +231,10 @@
     <xf numFmtId="0" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -252,11 +252,11 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1425,6 +1425,49 @@
           <order val="0"/>
           <tx>
             <strRef>
+              <f>'指标趋势'!B191</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln w="22000">
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="circle"/>
+            <size val="7"/>
+            <spPr>
+              <a:solidFill>
+                <a:srgbClr val="2E75B6"/>
+              </a:solidFill>
+              <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="2E75B6"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <xVal>
+            <numRef>
+              <f>'指标趋势'!$A$192:$A$193</f>
+            </numRef>
+          </xVal>
+          <yVal>
+            <numRef>
+              <f>'指标趋势'!$B$192:$B$193</f>
+            </numRef>
+          </yVal>
+          <smooth val="0"/>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
               <f>'指标趋势'!C191</f>
             </strRef>
           </tx>
@@ -1453,19 +1496,19 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'指标趋势'!$A$192</f>
+              <f>'指标趋势'!$A$192:$A$193</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'指标趋势'!$C$192</f>
+              <f>'指标趋势'!$C$192:$C$193</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="1"/>
-          <order val="1"/>
+          <idx val="2"/>
+          <order val="2"/>
           <tx>
             <strRef>
               <f>'指标趋势'!E191</f>
@@ -1500,8 +1543,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="2"/>
-          <order val="2"/>
+          <idx val="3"/>
+          <order val="3"/>
           <tx>
             <strRef>
               <f>'指标趋势'!G191</f>
@@ -1536,8 +1579,8 @@
           <smooth val="0"/>
         </ser>
         <ser>
-          <idx val="3"/>
-          <order val="3"/>
+          <idx val="4"/>
+          <order val="4"/>
           <tx>
             <strRef>
               <f>'指标趋势'!I191</f>
@@ -1579,7 +1622,7 @@
         <scaling>
           <orientation val="minMax"/>
           <max val="46309"/>
-          <min val="46307"/>
+          <min val="46308"/>
         </scaling>
         <delete val="0"/>
         <axPos val="l"/>
@@ -8522,7 +8565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J185"/>
+  <dimension ref="A1:J186"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8593,16 +8636,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.9565217391304348</v>
+        <v>0.9782608695652174</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>44/46</t>
+          <t>45/46</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 24/25 + 交付 20/21 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 25/25 + 交付 20/21 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8625,16 +8668,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.8032786885245902</v>
+        <v>0.819672131147541</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>49/61</t>
+          <t>50/61</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 16/24 + 交付 33/37 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 17/24 + 交付 33/37 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8657,16 +8700,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.7313432835820896</v>
+        <v>0.746268656716418</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>49/67</t>
+          <t>50/67</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 14/24 + 交付 35/43 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 15/24 + 交付 35/43 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8778,13 +8821,13 @@
         <v>46314</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.9565</v>
+        <v>0.9782999999999999</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0.8033</v>
+        <v>0.8197</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.7313</v>
+        <v>0.7463</v>
       </c>
     </row>
     <row r="12">
@@ -9818,51 +9861,51 @@
     </row>
     <row r="56">
       <c r="A56" s="17" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="B56" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>补录</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>KR4.2</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
+          <t>[V0差距] KR4.2 补录 2047 板上 12-bit(32 bit 像素) WiFi→PL 通路实测 (D15b 3a41eb7); V0 达成率 95.7%→97.8%, 仅剩 D29 冷上电 20 次</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1017_03_24h</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="17" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B57" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46313</v>
+      </c>
+      <c r="B57" s="6" t="inlineStr">
+        <is>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>D27</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
+          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/SPEC.md</t>
+          <t>progress/soak_v0/1017_03_24h</t>
         </is>
       </c>
     </row>
@@ -9870,24 +9913,24 @@
       <c r="A58" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B58" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>V2-5</t>
+          <t>D27</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
+          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_fmt/README.md</t>
+          <t>dr1v90 d27_link/SPEC.md</t>
         </is>
       </c>
     </row>
@@ -9902,17 +9945,17 @@
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>D28b</t>
+          <t>V2-5</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
+          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/回板当天.md</t>
+          <t>dr1v90 v2_fmt/README.md</t>
         </is>
       </c>
     </row>
@@ -9920,24 +9963,24 @@
       <c r="A60" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B60" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B60" s="6" t="inlineStr">
+        <is>
+          <t>进展</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>D27b</t>
+          <t>D28b</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
+          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/README.md</t>
+          <t>dr1v90 v1_bringup/回板当天.md</t>
         </is>
       </c>
     </row>
@@ -9945,24 +9988,24 @@
       <c r="A61" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B61" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B61" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>V2-6</t>
+          <t>D27b</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
+          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 gw5a_bridge/p2/README.md</t>
+          <t>dr1v90 d27_link/README.md</t>
         </is>
       </c>
     </row>
@@ -9972,22 +10015,22 @@
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>全套</t>
+          <t>V2-6</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
+          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ~/full_*.log</t>
+          <t>dr1v90 gw5a_bridge/p2/README.md</t>
         </is>
       </c>
     </row>
@@ -9997,22 +10040,22 @@
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>修复</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>全套</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
+          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 slice/SPEC.md §13.2</t>
+          <t>dr1v90 ~/full_*.log</t>
         </is>
       </c>
     </row>
@@ -10022,22 +10065,22 @@
       </c>
       <c r="B64" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
+          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1016_wkend_24h</t>
+          <t>dr1v90 slice/SPEC.md §13.2</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10090,7 @@
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -10057,37 +10100,37 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
+          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1017_*.log</t>
+          <t>progress/soak_v0/1016_wkend_24h</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>部署</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
+          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22c.board.log</t>
+          <t>progress/v0_accept/accept_1017_*.log</t>
         </is>
       </c>
     </row>
@@ -10095,9 +10138,9 @@
       <c r="A67" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B67" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
@@ -10107,12 +10150,12 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
+          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d22c.board.log</t>
         </is>
       </c>
     </row>
@@ -10120,24 +10163,24 @@
       <c r="A68" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B68" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B68" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
+          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board5.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10145,9 +10188,9 @@
       <c r="A69" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B69" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B69" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
@@ -10157,12 +10200,12 @@
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
+          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d21.board5.log</t>
         </is>
       </c>
     </row>
@@ -10177,12 +10220,12 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
+          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -10195,9 +10238,9 @@
       <c r="A71" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B71" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B71" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
@@ -10207,12 +10250,12 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
+          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_A fps_B</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10220,9 +10263,9 @@
       <c r="A72" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B72" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B72" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
@@ -10232,12 +10275,12 @@
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
+          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_C</t>
+          <t>soak_runs/fps_A fps_B</t>
         </is>
       </c>
     </row>
@@ -10245,24 +10288,24 @@
       <c r="A73" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B73" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B73" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
+          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20d-ackrps db4ec93</t>
+          <t>soak_runs/fps_C</t>
         </is>
       </c>
     </row>
@@ -10277,17 +10320,17 @@
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
+          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
+          <t>dr1v90 task/d20d-ackrps db4ec93</t>
         </is>
       </c>
     </row>
@@ -10297,22 +10340,22 @@
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
+          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_D</t>
+          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
         </is>
       </c>
     </row>
@@ -10320,9 +10363,9 @@
       <c r="A76" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
@@ -10332,12 +10375,12 @@
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
+          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>soak_runs/fps_D</t>
         </is>
       </c>
     </row>
@@ -10345,24 +10388,24 @@
       <c r="A77" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
+          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>~/rv_deploy.board.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10370,24 +10413,24 @@
       <c r="A78" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B78" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B78" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
+          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_deploy.board.log</t>
         </is>
       </c>
     </row>
@@ -10395,24 +10438,24 @@
       <c r="A79" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B79" s="6" t="inlineStr">
-        <is>
-          <t>验收</t>
+      <c r="B79" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
+          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10422,22 +10465,22 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>开工</t>
+          <t>验收</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>D20e/D23</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
+          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
+          <t>progress/v0_accept/</t>
         </is>
       </c>
     </row>
@@ -10445,24 +10488,24 @@
       <c r="A81" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B81" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B81" s="6" t="inlineStr">
+        <is>
+          <t>开工</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D24</t>
+          <t>D20e/D23</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
+          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>用户</t>
+          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
         </is>
       </c>
     </row>
@@ -10470,24 +10513,24 @@
       <c r="A82" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B82" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B82" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D24</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
+          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
@@ -10502,12 +10545,12 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
+          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -10520,24 +10563,24 @@
       <c r="A84" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
+          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1016_d20e.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10545,24 +10588,24 @@
       <c r="A85" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B85" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>KR7.3/D24</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
+          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/v0_accept/accept_1016_d20e.log</t>
         </is>
       </c>
     </row>
@@ -10570,24 +10613,24 @@
       <c r="A86" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B86" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B86" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>KR7.3/D24</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
+          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
         <is>
-          <t>D:\card03</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10595,24 +10638,24 @@
       <c r="A87" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B87" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B87" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>D25</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
+          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>D:\card03</t>
         </is>
       </c>
     </row>
@@ -10620,24 +10663,24 @@
       <c r="A88" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B88" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B88" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D25</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
+          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\cap_COM29.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10652,17 +10695,17 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
+          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20d_ackrps d20c_fps</t>
+          <t>D:\card03\cap_COM29.log</t>
         </is>
       </c>
     </row>
@@ -10670,24 +10713,24 @@
       <c r="A90" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B90" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B90" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
+          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d12_latency/RESULTS.md</t>
+          <t>dr1v90 d20d_ackrps d20c_fps</t>
         </is>
       </c>
     </row>
@@ -10702,17 +10745,17 @@
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
+          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d9_e2e/</t>
+          <t>dr1v90 d12_latency/RESULTS.md</t>
         </is>
       </c>
     </row>
@@ -10720,24 +10763,24 @@
       <c r="A92" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B92" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B92" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
+          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\boot03.log</t>
+          <t>dr1v90 d9_e2e/</t>
         </is>
       </c>
     </row>
@@ -10745,24 +10788,24 @@
       <c r="A93" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B93" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B93" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>D26</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
+          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
+          <t>D:\card03\boot03.log</t>
         </is>
       </c>
     </row>
@@ -10770,24 +10813,24 @@
       <c r="A94" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B94" s="6" t="inlineStr">
-        <is>
-          <t>开工</t>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>周末</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
+          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
+          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
         </is>
       </c>
     </row>
@@ -10797,22 +10840,22 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>方案</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>D29</t>
+          <t>周末</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
+          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d29_sdboot/PLAN.md</t>
+          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
         </is>
       </c>
     </row>
@@ -10820,24 +10863,24 @@
       <c r="A96" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B96" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B96" s="6" t="inlineStr">
+        <is>
+          <t>方案</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D28</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
+          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/</t>
+          <t>dr1v90 d29_sdboot/PLAN.md</t>
         </is>
       </c>
     </row>
@@ -10845,24 +10888,24 @@
       <c r="A97" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B97" s="6" t="inlineStr">
-        <is>
-          <t>修复</t>
+      <c r="B97" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>D30</t>
+          <t>D28</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
+          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
+          <t>dr1v90 v1_bringup/</t>
         </is>
       </c>
     </row>
@@ -10872,22 +10915,22 @@
       </c>
       <c r="B98" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>V2-3</t>
+          <t>D30</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
+          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_map/DESIGN.md</t>
+          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
         </is>
       </c>
     </row>
@@ -10897,47 +10940,47 @@
       </c>
       <c r="B99" s="6" t="inlineStr">
         <is>
-          <t>评估</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>V2-3</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
+          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d31_v1odd/REPORT.md</t>
+          <t>dr1v90 v2_map/DESIGN.md</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B100" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B100" s="6" t="inlineStr">
+        <is>
+          <t>评估</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>dr1v90 d31_v1odd/REPORT.md</t>
         </is>
       </c>
     </row>
@@ -10945,24 +10988,24 @@
       <c r="A101" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B101" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -10977,17 +11020,17 @@
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -10995,24 +11038,24 @@
       <c r="A103" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B103" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -11027,12 +11070,12 @@
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
@@ -11045,24 +11088,24 @@
       <c r="A105" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B105" s="6" t="inlineStr">
-        <is>
-          <t>分析</t>
+      <c r="B105" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11070,24 +11113,24 @@
       <c r="A106" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B106" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B106" s="6" t="inlineStr">
+        <is>
+          <t>分析</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -11095,19 +11138,19 @@
       <c r="A107" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B107" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
@@ -11120,24 +11163,24 @@
       <c r="A108" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B108" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -11145,24 +11188,24 @@
       <c r="A109" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B109" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B109" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -11170,24 +11213,24 @@
       <c r="A110" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B110" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -11202,17 +11245,17 @@
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -11222,22 +11265,22 @@
       </c>
       <c r="B112" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -11245,24 +11288,24 @@
       <c r="A113" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B113" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B113" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -11270,24 +11313,24 @@
       <c r="A114" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B114" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B114" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11297,22 +11340,22 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -11320,24 +11363,24 @@
       <c r="A116" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B116" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -11345,9 +11388,9 @@
       <c r="A117" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B117" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B117" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
@@ -11357,12 +11400,12 @@
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11377,17 +11420,17 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -11397,7 +11440,7 @@
       </c>
       <c r="B119" s="6" t="inlineStr">
         <is>
-          <t>复验</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
@@ -11407,12 +11450,12 @@
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -11422,22 +11465,22 @@
       </c>
       <c r="B120" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>复验</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -11445,9 +11488,9 @@
       <c r="A121" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B121" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B121" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
@@ -11457,12 +11500,12 @@
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -11470,24 +11513,24 @@
       <c r="A122" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B122" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B122" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11495,24 +11538,24 @@
       <c r="A123" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B123" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B123" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -11527,17 +11570,17 @@
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -11557,7 +11600,7 @@
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
@@ -11570,9 +11613,9 @@
       <c r="A126" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
@@ -11582,12 +11625,12 @@
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -11597,22 +11640,22 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
@@ -11627,17 +11670,17 @@
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
@@ -11647,7 +11690,7 @@
       </c>
       <c r="B129" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
@@ -11657,12 +11700,12 @@
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
@@ -11672,7 +11715,7 @@
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
@@ -11682,12 +11725,12 @@
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
@@ -11697,47 +11740,47 @@
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B132" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B132" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -11745,24 +11788,24 @@
       <c r="A133" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B133" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -11770,24 +11813,24 @@
       <c r="A134" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B134" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B134" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -11807,7 +11850,7 @@
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
@@ -11820,24 +11863,24 @@
       <c r="A136" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B136" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B136" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -11845,24 +11888,24 @@
       <c r="A137" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B137" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B137" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -11870,9 +11913,9 @@
       <c r="A138" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B138" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B138" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
@@ -11882,12 +11925,12 @@
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -11895,9 +11938,9 @@
       <c r="A139" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B139" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B139" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
@@ -11907,12 +11950,12 @@
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -11920,24 +11963,24 @@
       <c r="A140" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B140" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B140" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -11945,24 +11988,24 @@
       <c r="A141" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B141" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B141" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -11970,24 +12013,24 @@
       <c r="A142" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B142" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B142" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -11995,24 +12038,24 @@
       <c r="A143" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B143" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B143" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -12020,9 +12063,9 @@
       <c r="A144" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B144" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B144" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
@@ -12032,12 +12075,12 @@
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -12045,24 +12088,24 @@
       <c r="A145" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B145" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B145" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -12070,9 +12113,9 @@
       <c r="A146" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B146" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B146" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
@@ -12082,12 +12125,12 @@
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12095,24 +12138,24 @@
       <c r="A147" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B147" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B147" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -12120,24 +12163,24 @@
       <c r="A148" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B148" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B148" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12145,24 +12188,24 @@
       <c r="A149" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B149" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B149" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -12170,24 +12213,24 @@
       <c r="A150" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B150" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B150" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -12195,24 +12238,24 @@
       <c r="A151" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B151" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B151" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
@@ -12220,24 +12263,24 @@
       <c r="A152" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B152" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B152" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
@@ -12245,49 +12288,49 @@
       <c r="A153" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B153" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B154" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B154" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -12302,17 +12345,17 @@
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -12327,17 +12370,17 @@
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -12345,9 +12388,9 @@
       <c r="A157" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B157" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B157" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
@@ -12357,12 +12400,12 @@
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -12370,9 +12413,9 @@
       <c r="A158" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B158" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B158" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C158" s="7" t="inlineStr">
@@ -12382,12 +12425,12 @@
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -12395,24 +12438,24 @@
       <c r="A159" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B159" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B159" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -12420,9 +12463,9 @@
       <c r="A160" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B160" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B160" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C160" s="7" t="inlineStr">
@@ -12432,12 +12475,12 @@
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12452,17 +12495,17 @@
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -12470,9 +12513,9 @@
       <c r="A162" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B162" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B162" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C162" s="7" t="inlineStr">
@@ -12482,12 +12525,12 @@
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -12507,7 +12550,7 @@
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
@@ -12520,24 +12563,24 @@
       <c r="A164" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B164" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B164" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E164" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12545,24 +12588,24 @@
       <c r="A165" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B165" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B165" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -12570,24 +12613,24 @@
       <c r="A166" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B166" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B166" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C166" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E166" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12602,17 +12645,17 @@
       </c>
       <c r="C167" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -12620,19 +12663,19 @@
       <c r="A168" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B168" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B168" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C168" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E168" s="7" t="inlineStr">
@@ -12645,9 +12688,9 @@
       <c r="A169" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B169" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B169" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C169" s="7" t="inlineStr">
@@ -12657,12 +12700,12 @@
       </c>
       <c r="D169" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12670,24 +12713,24 @@
       <c r="A170" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B170" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B170" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C170" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -12695,9 +12738,9 @@
       <c r="A171" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B171" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B171" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C171" s="7" t="inlineStr">
@@ -12707,12 +12750,12 @@
       </c>
       <c r="D171" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12720,9 +12763,9 @@
       <c r="A172" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B172" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B172" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C172" s="7" t="inlineStr">
@@ -12732,12 +12775,12 @@
       </c>
       <c r="D172" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -12745,24 +12788,24 @@
       <c r="A173" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B173" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B173" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C173" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12770,24 +12813,24 @@
       <c r="A174" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B174" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B174" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C174" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E174" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -12800,15 +12843,19 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C175" s="7" t="inlineStr"/>
+      <c r="C175" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12816,15 +12863,15 @@
       <c r="A176" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B176" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B176" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C176" s="7" t="inlineStr"/>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E176" s="7" t="inlineStr">
@@ -12837,20 +12884,20 @@
       <c r="A177" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B177" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B177" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C177" s="7" t="inlineStr"/>
       <c r="D177" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -12863,19 +12910,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C178" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="C178" s="7" t="inlineStr"/>
       <c r="D178" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -12890,12 +12933,12 @@
       </c>
       <c r="C179" s="7" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D179" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
@@ -12915,12 +12958,12 @@
       </c>
       <c r="C180" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E180" s="7" t="inlineStr">
@@ -12940,12 +12983,12 @@
       </c>
       <c r="C181" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
@@ -12965,12 +13008,12 @@
       </c>
       <c r="C182" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D182" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E182" s="7" t="inlineStr">
@@ -12990,17 +13033,17 @@
       </c>
       <c r="C183" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D15;D16</t>
         </is>
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13008,24 +13051,24 @@
       <c r="A184" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B184" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B184" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C184" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>KR5.2</t>
         </is>
       </c>
       <c r="D184" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
         </is>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 49031f6</t>
         </is>
       </c>
     </row>
@@ -13033,18 +13076,43 @@
       <c r="A185" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B185" s="19" t="inlineStr">
+      <c r="B185" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C185" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D185" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E185" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B186" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C185" s="7" t="inlineStr"/>
-      <c r="D185" s="7" t="inlineStr">
+      <c r="C186" s="7" t="inlineStr"/>
+      <c r="D186" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E185" s="7" t="inlineStr">
+      <c r="E186" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -13818,9 +13886,9 @@
           <t>显示优化</t>
         </is>
       </c>
-      <c r="D14" s="24" t="inlineStr">
-        <is>
-          <t>⏸ 无数据 / 未开始</t>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>✅ 达成当前期目标</t>
         </is>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -13906,11 +13974,11 @@
         <v>1</v>
       </c>
       <c r="J15" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>仿真</t>
+          <t>V0 2047</t>
         </is>
       </c>
       <c r="L15" s="6" t="n">
@@ -13922,14 +13990,14 @@
       <c r="N15" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="O15" s="24" t="inlineStr">
-        <is>
-          <t>⏸</t>
+      <c r="O15" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="P15" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8 (D15 阶段 1, 主会话复验)</t>
+          <t>dr1v90 3a41eb7 (D15b 主会话新克隆上板复验; V0 出口⑦ 10-14 daily_log)</t>
         </is>
       </c>
       <c r="Q15" s="21" t="n">
@@ -14839,7 +14907,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="A31" s="24" t="inlineStr">
         <is>
           <t>图例</t>
         </is>
@@ -14851,7 +14919,7 @@
           <t>✅</t>
         </is>
       </c>
-      <c r="B32" s="26" t="inlineStr">
+      <c r="B32" s="25" t="inlineStr">
         <is>
           <t>达成当前期目标</t>
         </is>
@@ -14863,19 +14931,19 @@
           <t>🔄</t>
         </is>
       </c>
-      <c r="B33" s="26" t="inlineStr">
+      <c r="B33" s="25" t="inlineStr">
         <is>
           <t>进行中 / 未达标</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
+      <c r="A34" s="26" t="inlineStr">
         <is>
           <t>⏸</t>
         </is>
       </c>
-      <c r="B34" s="26" t="inlineStr">
+      <c r="B34" s="25" t="inlineStr">
         <is>
           <t>无数据 / 未开始</t>
         </is>
@@ -14887,7 +14955,7 @@
           <t>❌</t>
         </is>
       </c>
-      <c r="B35" s="26" t="inlineStr">
+      <c r="B35" s="25" t="inlineStr">
         <is>
           <t>退步 / 阻塞</t>
         </is>
@@ -16279,25 +16347,32 @@
         <v>1</v>
       </c>
       <c r="D192" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="E192" s="6" t="n">
         <v>1</v>
       </c>
       <c r="F192" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="G192" s="6" t="n">
         <v>1</v>
       </c>
       <c r="H192" s="8" t="n">
-        <v>46307</v>
+        <v>46308</v>
       </c>
       <c r="I192" s="6" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="193">
+      <c r="A193" s="8" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B193" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="C193" s="6" t="n"/>
       <c r="D193" s="8" t="n">
         <v>46309</v>
       </c>
@@ -18688,7 +18763,7 @@
         <v>46319</v>
       </c>
       <c r="F42" s="17" t="n"/>
-      <c r="G42" s="24" t="inlineStr">
+      <c r="G42" s="26" t="inlineStr">
         <is>
           <t>⏸</t>
         </is>
@@ -18912,7 +18987,7 @@
       </c>
       <c r="E48" s="17" t="n"/>
       <c r="F48" s="17" t="n"/>
-      <c r="G48" s="24" t="inlineStr">
+      <c r="G48" s="26" t="inlineStr">
         <is>
           <t>⏸</t>
         </is>
@@ -18946,7 +19021,7 @@
       </c>
       <c r="E49" s="17" t="n"/>
       <c r="F49" s="17" t="n"/>
-      <c r="G49" s="24" t="inlineStr">
+      <c r="G49" s="26" t="inlineStr">
         <is>
           <t>⏸</t>
         </is>
@@ -19016,7 +19091,7 @@
       </c>
       <c r="E51" s="17" t="n"/>
       <c r="F51" s="17" t="n"/>
-      <c r="G51" s="24" t="inlineStr">
+      <c r="G51" s="26" t="inlineStr">
         <is>
           <t>⏸</t>
         </is>
@@ -19839,7 +19914,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="25" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>对角线 (y = x)</t>
         </is>
@@ -19873,7 +19948,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I79"/>
+  <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -22686,25 +22761,25 @@
         <v>46309</v>
       </c>
       <c r="B69" s="7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>KR7.1</t>
+          <t>KR4.2</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>丢帧/迟到率</t>
+          <t>链路色深 12-bit 已验证 (1=是)</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>是/否</t>
         </is>
       </c>
       <c r="F69" s="7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G69" s="7" t="inlineStr">
         <is>
@@ -22713,12 +22788,12 @@
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3 (主会话上板复验 v4.log)</t>
+          <t>dr1v90 3a41eb7 (D15b 主会话新克隆上板复验; V0 出口⑦ 10-14 daily_log)</t>
         </is>
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片 60 min 带载: late 0 / miss 0 (按片); drop 为显示自身跳角, 不计</t>
+          <t>补录 [V0差距]: 2047 板上 32 bit 像素 X2R10G10B10 与 16 bit 路径 PL==CPU 逐字节, 32 bit 推流 PL @10.83 rps 600 s 完成率 100%; 仅覆盖 WiFi→板端 PL 段, 板→2260 LVDS 段仍是仿真 (D5/D8/D9), 如认为 KR4.2 须含 LVDS 段请撤销此行</t>
         </is>
       </c>
     </row>
@@ -22731,21 +22806,21 @@
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>KR7.1</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>连续无故障: 软件链路 (假转, 无人值守)</t>
+          <t>丢帧/迟到率</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F70" s="7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G70" s="7" t="inlineStr">
         <is>
@@ -22754,12 +22829,12 @@
       </c>
       <c r="H70" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/pls-2047 782e9e3 (主会话上板复验 v4.log)</t>
         </is>
       </c>
       <c r="I70" s="7" t="inlineStr">
         <is>
-          <t>假转无人值守带载连续 60 min 无停摆无错 (目标 8 h, 未达)</t>
+          <t>2047 PL 切片 60 min 带载: late 0 / miss 0 (按片); drop 为显示自身跳角, 不计</t>
         </is>
       </c>
     </row>
@@ -22768,25 +22843,25 @@
         <v>46309</v>
       </c>
       <c r="B71" s="7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>KR8.1</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>上电到 0° 片亮起 (停转)</t>
+          <t>连续无故障: 软件链路 (假转, 无人值守)</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>s</t>
+          <t>h</t>
         </is>
       </c>
       <c r="F71" s="7" t="n">
-        <v>17.2</v>
+        <v>1</v>
       </c>
       <c r="G71" s="7" t="inlineStr">
         <is>
@@ -22795,12 +22870,12 @@
       </c>
       <c r="H71" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4 (上板 3 次重启 17.17–17.30 s)</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
       <c r="I71" s="7" t="inlineStr">
         <is>
-          <t>PL 默认开机 (多加载 PL 位流), 从 reboot 命令算</t>
+          <t>假转无人值守带载连续 60 min 无停摆无错 (目标 8 h, 未达)</t>
         </is>
       </c>
     </row>
@@ -22827,7 +22902,7 @@
         </is>
       </c>
       <c r="F72" s="7" t="n">
-        <v>12.4</v>
+        <v>17.2</v>
       </c>
       <c r="G72" s="7" t="inlineStr">
         <is>
@@ -22836,12 +22911,12 @@
       </c>
       <c r="H72" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d13_boot/runs/20261014_145507 (串口 3 次)</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4 (上板 3 次重启 17.17–17.30 s)</t>
         </is>
       </c>
       <c r="I72" s="7" t="inlineStr">
         <is>
-          <t>D13 第二步后 (bootdelay 0 + 精简 uInitrd) + PL 默认开机</t>
+          <t>PL 默认开机 (多加载 PL 位流), 从 reboot 命令算</t>
         </is>
       </c>
     </row>
@@ -22854,12 +22929,12 @@
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>KR8.2</t>
+          <t>KR8.1</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>按名字找到板子</t>
+          <t>上电到 0° 片亮起 (停转)</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
@@ -22868,7 +22943,7 @@
         </is>
       </c>
       <c r="F73" s="7" t="n">
-        <v>24.4</v>
+        <v>12.4</v>
       </c>
       <c r="G73" s="7" t="inlineStr">
         <is>
@@ -22877,12 +22952,12 @@
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>dr1v90 d13_boot/runs/20261014_145507 (串口 3 次)</t>
         </is>
       </c>
       <c r="I73" s="7" t="inlineStr">
         <is>
-          <t>PL 默认开机找板 24.4–28.3 s</t>
+          <t>D13 第二步后 (bootdelay 0 + 精简 uInitrd) + PL 默认开机</t>
         </is>
       </c>
     </row>
@@ -22909,7 +22984,7 @@
         </is>
       </c>
       <c r="F74" s="7" t="n">
-        <v>19.8</v>
+        <v>24.4</v>
       </c>
       <c r="G74" s="7" t="inlineStr">
         <is>
@@ -22918,12 +22993,12 @@
       </c>
       <c r="H74" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d13_boot/runs/20261014_145507</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
       <c r="I74" s="7" t="inlineStr">
         <is>
-          <t>3 次 19.8/20.3/20.9 s</t>
+          <t>PL 默认开机找板 24.4–28.3 s</t>
         </is>
       </c>
     </row>
@@ -22932,25 +23007,25 @@
         <v>46309</v>
       </c>
       <c r="B75" s="7" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>KR9.1</t>
+          <t>KR8.2</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>转子遥测可用 (1=可用)</t>
+          <t>按名字找到板子</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>是/否</t>
+          <t>s</t>
         </is>
       </c>
       <c r="F75" s="7" t="n">
-        <v>1</v>
+        <v>19.8</v>
       </c>
       <c r="G75" s="7" t="inlineStr">
         <is>
@@ -22959,12 +23034,12 @@
       </c>
       <c r="H75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>dr1v90 d13_boot/runs/20261014_145507</t>
         </is>
       </c>
       <c r="I75" s="7" t="inlineStr">
         <is>
-          <t>povstat 遥测 + povnetd 状态上板可用</t>
+          <t>3 次 19.8/20.3/20.9 s</t>
         </is>
       </c>
     </row>
@@ -22977,12 +23052,12 @@
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>KR9.2</t>
+          <t>KR9.1</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>远程升级失败自动回滚 (1=有)</t>
+          <t>转子遥测可用 (1=可用)</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -23005,34 +23080,34 @@
       </c>
       <c r="I76" s="7" t="inlineStr">
         <is>
-          <t>断网坏升级包连续 3 次自动回滚并按名字找回; 坏自检包回滚</t>
+          <t>povstat 遥测 + povnetd 状态上板可用</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="29" t="n">
-        <v>46310</v>
+        <v>46309</v>
       </c>
       <c r="B77" s="7" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>KR7.1</t>
+          <t>KR9.2</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>丢帧/迟到率</t>
+          <t>远程升级失败自动回滚 (1=有)</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>是/否</t>
         </is>
       </c>
       <c r="F77" s="7" t="n">
-        <v>0.0012</v>
+        <v>1</v>
       </c>
       <c r="G77" s="7" t="inlineStr">
         <is>
@@ -23041,12 +23116,12 @@
       </c>
       <c r="H77" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fe53bde</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
       <c r="I77" s="7" t="inlineStr">
         <is>
-          <t>8 h 内最差一小时未完成片 0.0012% (每 10 s 窗口完成率均 100%)</t>
+          <t>断网坏升级包连续 3 次自动回滚并按名字找回; 坏自检包回滚</t>
         </is>
       </c>
     </row>
@@ -23059,21 +23134,21 @@
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>KR7.1</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>连续无故障: 软件链路 (假转, 无人值守)</t>
+          <t>丢帧/迟到率</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>%</t>
         </is>
       </c>
       <c r="F78" s="7" t="n">
-        <v>8</v>
+        <v>0.0012</v>
       </c>
       <c r="G78" s="7" t="inlineStr">
         <is>
@@ -23082,12 +23157,12 @@
       </c>
       <c r="H78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fe53bde; progress/soak_v0/report.md</t>
+          <t>dr1v90 fe53bde</t>
         </is>
       </c>
       <c r="I78" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守 (假转黑屏, 主线 voxslice 0.6 + PL 默认): 停摆 0 / 死 0 / 对拍 204/0 / 推流 14.65 fps 11 段 / ping 961 丢 0 / 内存不涨</t>
+          <t>8 h 内最差一小时未完成片 0.0012% (每 10 s 窗口完成率均 100%)</t>
         </is>
       </c>
     </row>
@@ -23100,40 +23175,81 @@
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
+          <t>KR7.2</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>连续无故障: 软件链路 (假转, 无人值守)</t>
+        </is>
+      </c>
+      <c r="E79" s="7" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="n">
+        <v>8</v>
+      </c>
+      <c r="G79" s="7" t="inlineStr">
+        <is>
+          <t>V0 2047</t>
+        </is>
+      </c>
+      <c r="H79" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 fe53bde; progress/soak_v0/report.md</t>
+        </is>
+      </c>
+      <c r="I79" s="7" t="inlineStr">
+        <is>
+          <t>8 h 无人值守 (假转黑屏, 主线 voxslice 0.6 + PL 默认): 停摆 0 / 死 0 / 对拍 204/0 / 推流 14.65 fps 11 段 / ping 961 丢 0 / 内存不涨</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="29" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B80" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C80" s="7" t="inlineStr">
+        <is>
           <t>KR7.3</t>
         </is>
       </c>
-      <c r="D79" s="7" t="inlineStr">
+      <c r="D80" s="7" t="inlineStr">
         <is>
           <t>连续无故障: 整机实转 (有人值守)</t>
         </is>
       </c>
-      <c r="E79" s="7" t="inlineStr">
+      <c r="E80" s="7" t="inlineStr">
         <is>
           <t>h</t>
         </is>
       </c>
-      <c r="F79" s="7" t="n">
+      <c r="F80" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="G79" s="7" t="inlineStr">
+      <c r="G80" s="7" t="inlineStr">
         <is>
           <t>V0 2047</t>
         </is>
       </c>
-      <c r="H79" s="7" t="inlineStr">
+      <c r="H80" s="7" t="inlineStr">
         <is>
           <t>progress/realspin_v0/</t>
         </is>
       </c>
-      <c r="I79" s="7" t="inlineStr">
+      <c r="I80" s="7" t="inlineStr">
         <is>
           <t>实转 583 rpm 1 h (有人值守, 开机默认 PL + QoS 开): 停摆 0 / 死 0 / NAK 0 / ERR 0 / 转动 57/57 min / ping 121 丢 0 / 完成率最低 99.84% (16 位回绕已补); 换帧 10.45/s 受转速限制 (D19 在修)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I79"/>
+  <autoFilter ref="A1:I80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
进度看板 10-19 更新: D33-D39/V2-7 完成, V0 97.8% / V1 85.3% / V2 79.7%
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-19.xlsx
+++ b/docs/progress/显性目的进度_2026-10-19.xlsx
@@ -8565,7 +8565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J186"/>
+  <dimension ref="A1:J201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8668,16 +8668,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.819672131147541</v>
+        <v>0.8529411764705882</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>50/61</t>
+          <t>58/68</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 17/24 + 交付 33/37 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 17/24 + 交付 41/44 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8700,16 +8700,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.746268656716418</v>
+        <v>0.7972972972972973</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>50/67</t>
+          <t>59/74</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 15/24 + 交付 35/43 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 15/24 + 交付 44/50 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8824,10 +8824,10 @@
         <v>0.9782999999999999</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0.8197</v>
+        <v>0.8529</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.7463</v>
+        <v>0.7973</v>
       </c>
     </row>
     <row r="12">
@@ -9886,586 +9886,586 @@
     </row>
     <row r="57">
       <c r="A57" s="17" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="B57" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>V1</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
+          <t>用户确认: SoC 底板 10-15 与桥转接板 10-16 都已投板 (11-10 回板即此版), 不能改图; 软件此前依据 10-12 版 → 开 D36 按新版网表全面对齐, 需硬件改动一律写回板后改板清单; D35 (W6/面 B) 同口径; 新版文件集中在 hw_latest_1016/</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1017_03_24h</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="17" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B58" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46314</v>
+      </c>
+      <c r="B58" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
         <is>
-          <t>D27</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
+          <t>03 软重启 20/20 进内核+回网 (串口录制换自动重连 cap2.ps1, 旧录制掉电后句柄失效 0 字节); 冷上电改由 USB 继电器 (LCUS-1, 常闭串 24V+) 自动做, 用户已同意采购, 到货后验 20 次</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/SPEC.md</t>
+          <t>dr1v90 card03</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="17" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B59" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>合并</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>V2-5</t>
+          <t>D35</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
+          <t>V1 可装 A/B 两面 (W6=面B TXP7 非光电, 光电 CN3-R82-U12); 位流待改 spin_sync→U12、删 bank11 2047 屏脚; 主会话独立机读网表复核一致</t>
         </is>
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_fmt/README.md</t>
+          <t>dr1v90 2b111f0</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="17" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B60" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>D28b</t>
+          <t>D36</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
+          <t>投板版网表对齐: 唯一引脚变化 UL_CHK→R7/T7, 光电 W6→U12, CN3/CN6 101-n 正确 (B3 作废); 改约束已入 task/d36-hwsync 42eca66; 位流重出待用户放行; 回板当天改板清单 PDF 出</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/回板当天.md</t>
+          <t>docs progress/回板当天改板清单_2026-10-19.pdf</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="17" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B61" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46314</v>
+      </c>
+      <c r="B61" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
-          <t>D27b</t>
+          <t>D37</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
+          <t>用户定: V1 主控 bank33 走 1.8V (LVDS18), 桥板方案 A (U18/U19 VCCA 改 1.8V LDO, R236 NC); 底板 100Ω 空贴已确认; R82 改 5.6k; 桥 R235/R223 推荐 2.2k; 改板清单 PDF 已更新</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/README.md</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="17" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B62" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>V2-6</t>
+          <t>D36</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
+          <t>桥位流四套按投板版重出 (用户放行): e60c 7f612855 / e60p8c d93495b3 / e60 4c74afd7 / e60p8 7bd1967e, 0 违例; task/d36-hwsync 97a10cf 复验中</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 gw5a_bridge/p2/README.md</t>
+          <t>dr1v90 97a10cf</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="17" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B63" s="6" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>合并</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
-          <t>全套</t>
+          <t>D34</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
+          <t>V1 357/285/209 奇数档 + 24 Hz 满档; 复验 d25/d23/v1_bringup/d9 全过</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ~/full_*.log</t>
+          <t>dr1v90 7253608</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="17" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B64" s="6" t="inlineStr">
-        <is>
-          <t>修复</t>
+        <v>46314</v>
+      </c>
+      <c r="B64" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>D37</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
+          <t>用户改回: V1 主控 bank33 走 2.5V (H7/H9 专供 J1/J2), 桥板不改; R82 改 2.2k; 1.8V 方案不采用 (备查 d37_io18)</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 slice/SPEC.md §13.2</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="17" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B65" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>合并</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D33</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
+          <t>主控 JTAG 灌桥 (bringup --bridge-load sram, 盲灌+JT01-06 判据); 复验 53/0, v1_bringup 96/0</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1016_wkend_24h</t>
+          <t>dr1v90 23474c7</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="17" t="n">
-        <v>46312</v>
+        <v>46314</v>
       </c>
       <c r="B66" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>合并</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D36</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
+          <t>软件对齐投板版; 桥位流四套重出 0 违例</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1017_*.log</t>
+          <t>dr1v90 f2584d9</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="17" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="B67" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>合并</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D38</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
+          <t>V1 面 B 软件就绪 (IO 电压开关/面 B RTL/桥 B/JTAG 两器件链/--faces AB); 面 B 桥 e60cb f919ea30; 双面主控首建 TD 崩溃 (资源 74%, 拥塞), 重跑中</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22c.board.log</t>
+          <t>dr1v90 ad201f9</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B68" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46314</v>
+      </c>
+      <c r="B68" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>V1主控</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
+          <t>V1 单面主控位流 io25 2b4f3311 (光电 U12, 时序过), io18 备用 6493e837; _work/v1_main_1019</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>本机构建</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="17" t="n">
-        <v>46311</v>
+        <v>46314</v>
       </c>
       <c r="B69" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D39</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
+          <t>SoC↔桥通信专项验证包 comm_check.sh (不接屏, 自动判 PRBS/边带/寄存器/JTAG/恢复, 13 电平测点); 离线 88/0; 与 D38 冲突由 D39b 合并并出 PRBS 位流; 到板页 progress/到板当天_通信验证.pdf</t>
         </is>
       </c>
       <c r="E69" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board5.log</t>
+          <t>dr1v90 task/d39-comm b69f6d8</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B70" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46314</v>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>合并</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>V2-7</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
+          <t>板端 voxslice_p2 驱动 2 期主控 (--disp p2), 端到端逐像素 0 错, V0/V1 行为不变; regress 27/0</t>
         </is>
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 ff1846a</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B71" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46314</v>
+      </c>
+      <c r="B71" s="6" t="inlineStr">
+        <is>
+          <t>合并</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D39</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
+          <t>通信验证包进主线 + PRBS 位流 (桥 e60cp 6d5b3db3 / 主控 sb_prbs_io25 e7c33e78, 0 违例); 到板即可 comm_check.sh --board &lt;名&gt; --bridge-load sram; 复验 85/0 110/0 76/0</t>
         </is>
       </c>
       <c r="E71" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 3ef6b06</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="17" t="n">
-        <v>46311</v>
+        <v>46313</v>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>测量</t>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
+          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_A fps_B</t>
+          <t>progress/soak_v0/1017_03_24h</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B73" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46312</v>
+      </c>
+      <c r="B73" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D27</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
+          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_C</t>
+          <t>dr1v90 d27_link/SPEC.md</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B74" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>V2-5</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
+          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20d-ackrps db4ec93</t>
+          <t>dr1v90 v2_fmt/README.md</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B75" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D28b</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
+          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
+          <t>dr1v90 v1_bringup/回板当天.md</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B76" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+        <v>46312</v>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D27b</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
+          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_D</t>
+          <t>dr1v90 d27_link/README.md</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B77" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46312</v>
+      </c>
+      <c r="B77" s="6" t="inlineStr">
+        <is>
+          <t>进展</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>V2-6</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
+          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 gw5a_bridge/p2/README.md</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>全套</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
+          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>~/rv_deploy.board.log</t>
+          <t>dr1v90 ~/full_*.log</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="17" t="n">
-        <v>46311</v>
-      </c>
-      <c r="B79" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46312</v>
+      </c>
+      <c r="B79" s="6" t="inlineStr">
+        <is>
+          <t>修复</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
+          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 slice/SPEC.md §13.2</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>验收</t>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
@@ -10475,37 +10475,37 @@
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
+          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/</t>
+          <t>progress/soak_v0/1016_wkend_24h</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>开工</t>
+          <t>部署</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>D20e/D23</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
+          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
+          <t>progress/v0_accept/accept_1017_*.log</t>
         </is>
       </c>
     </row>
@@ -10513,24 +10513,24 @@
       <c r="A82" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B82" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B82" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D24</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
+          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>用户</t>
+          <t>~/rv_d22c.board.log</t>
         </is>
       </c>
     </row>
@@ -10545,12 +10545,12 @@
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
+          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -10563,24 +10563,24 @@
       <c r="A84" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B84" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B84" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
+          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d21.board5.log</t>
         </is>
       </c>
     </row>
@@ -10588,24 +10588,24 @@
       <c r="A85" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B85" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B85" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
+          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1016_d20e.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10620,12 +10620,12 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>KR7.3/D24</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
+          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
@@ -10640,22 +10640,22 @@
       </c>
       <c r="B87" s="6" t="inlineStr">
         <is>
-          <t>硬件</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
+          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>D:\card03</t>
+          <t>soak_runs/fps_A fps_B</t>
         </is>
       </c>
     </row>
@@ -10663,24 +10663,24 @@
       <c r="A88" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B88" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B88" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>D25</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
+          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>soak_runs/fps_C</t>
         </is>
       </c>
     </row>
@@ -10688,24 +10688,24 @@
       <c r="A89" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B89" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B89" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
+          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\cap_COM29.log</t>
+          <t>dr1v90 task/d20d-ackrps db4ec93</t>
         </is>
       </c>
     </row>
@@ -10713,24 +10713,24 @@
       <c r="A90" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B90" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B90" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
+          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20d_ackrps d20c_fps</t>
+          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
         </is>
       </c>
     </row>
@@ -10738,24 +10738,24 @@
       <c r="A91" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B91" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B91" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
+          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d12_latency/RESULTS.md</t>
+          <t>soak_runs/fps_D</t>
         </is>
       </c>
     </row>
@@ -10770,17 +10770,17 @@
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
+          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d9_e2e/</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10790,22 +10790,22 @@
       </c>
       <c r="B93" s="6" t="inlineStr">
         <is>
-          <t>硬件</t>
+          <t>部署</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
+          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\boot03.log</t>
+          <t>~/rv_deploy.board.log</t>
         </is>
       </c>
     </row>
@@ -10820,17 +10820,17 @@
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D26</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
+          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10840,22 +10840,22 @@
       </c>
       <c r="B95" s="6" t="inlineStr">
         <is>
-          <t>开工</t>
+          <t>验收</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>周末</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
+          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
+          <t>progress/v0_accept/</t>
         </is>
       </c>
     </row>
@@ -10865,22 +10865,22 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>方案</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D29</t>
+          <t>D20e/D23</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
+          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d29_sdboot/PLAN.md</t>
+          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
         </is>
       </c>
     </row>
@@ -10888,24 +10888,24 @@
       <c r="A97" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B97" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B97" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>D28</t>
+          <t>D24</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
+          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
@@ -10913,24 +10913,24 @@
       <c r="A98" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B98" s="6" t="inlineStr">
-        <is>
-          <t>修复</t>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>D30</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
+          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10938,24 +10938,24 @@
       <c r="A99" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B99" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>V2-3</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
+          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_map/DESIGN.md</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10965,28 +10965,28 @@
       </c>
       <c r="B100" s="6" t="inlineStr">
         <is>
-          <t>评估</t>
+          <t>部署</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
+          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d31_v1odd/REPORT.md</t>
+          <t>progress/v0_accept/accept_1016_d20e.log</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
@@ -10995,148 +10995,148 @@
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>KR7.3/D24</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B102" s="6" t="inlineStr">
         <is>
-          <t>测量</t>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>D:\card03</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B103" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+        <v>46311</v>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>D25</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B104" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46311</v>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>D:\card03\cap_COM29.log</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B105" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46311</v>
+      </c>
+      <c r="B105" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 d20d_ackrps d20c_fps</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B106" s="6" t="inlineStr">
-        <is>
-          <t>分析</t>
+        <v>46311</v>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>dr1v90 d12_latency/RESULTS.md</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
@@ -11145,217 +11145,217 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>dr1v90 d9_e2e/</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B108" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46311</v>
+      </c>
+      <c r="B108" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>D:\card03\boot03.log</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B109" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+        <v>46311</v>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B110" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B110" s="6" t="inlineStr">
+        <is>
+          <t>开工</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>周末</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>方案</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>dr1v90 d29_sdboot/PLAN.md</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B112" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+        <v>46311</v>
+      </c>
+      <c r="B112" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D28</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>dr1v90 v1_bringup/</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B113" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D30</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B114" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B114" s="6" t="inlineStr">
+        <is>
+          <t>进展</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>V2-3</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 v2_map/DESIGN.md</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="17" t="n">
-        <v>46310</v>
+        <v>46311</v>
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>评估</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 d31_v1odd/REPORT.md</t>
         </is>
       </c>
     </row>
@@ -11363,24 +11363,24 @@
       <c r="A116" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B116" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B116" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -11388,24 +11388,24 @@
       <c r="A117" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B117" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B117" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -11415,22 +11415,22 @@
       </c>
       <c r="B118" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>测量</t>
         </is>
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -11438,24 +11438,24 @@
       <c r="A119" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B119" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B119" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11463,24 +11463,24 @@
       <c r="A120" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B120" s="6" t="inlineStr">
-        <is>
-          <t>复验</t>
+      <c r="B120" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11490,22 +11490,22 @@
       </c>
       <c r="B121" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>分析</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -11520,17 +11520,17 @@
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -11538,24 +11538,24 @@
       <c r="A123" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B123" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B123" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -11563,24 +11563,24 @@
       <c r="A124" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B124" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B124" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -11588,24 +11588,24 @@
       <c r="A125" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B125" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -11613,24 +11613,24 @@
       <c r="A126" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B126" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B126" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -11640,22 +11640,22 @@
       </c>
       <c r="B127" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -11665,22 +11665,22 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -11688,24 +11688,24 @@
       <c r="A129" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B129" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11715,22 +11715,22 @@
       </c>
       <c r="B130" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -11740,22 +11740,22 @@
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -11763,230 +11763,230 @@
       <c r="A132" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B132" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B132" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B133" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B133" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B134" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46310</v>
+      </c>
+      <c r="B134" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B135" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B135" s="6" t="inlineStr">
+        <is>
+          <t>复验</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B136" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B136" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B137" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46310</v>
+      </c>
+      <c r="B137" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B138" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46310</v>
+      </c>
+      <c r="B138" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B139" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46310</v>
+      </c>
+      <c r="B139" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B140" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B140" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="17" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
       <c r="B141" s="15" t="inlineStr">
         <is>
@@ -11995,167 +11995,167 @@
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B142" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46310</v>
+      </c>
+      <c r="B142" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B143" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+        <v>46310</v>
+      </c>
+      <c r="B143" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B144" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46310</v>
+      </c>
+      <c r="B144" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B145" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+        <v>46310</v>
+      </c>
+      <c r="B145" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B146" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+        <v>46310</v>
+      </c>
+      <c r="B146" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B147" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46310</v>
+      </c>
+      <c r="B147" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -12163,24 +12163,24 @@
       <c r="A148" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B148" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B148" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -12188,24 +12188,24 @@
       <c r="A149" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B149" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B149" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -12213,24 +12213,24 @@
       <c r="A150" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B150" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B150" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -12238,24 +12238,24 @@
       <c r="A151" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B151" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B151" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -12263,24 +12263,24 @@
       <c r="A152" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B152" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B152" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -12288,24 +12288,24 @@
       <c r="A153" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B153" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B153" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -12313,399 +12313,399 @@
       <c r="A154" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B154" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B154" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B155" s="11" t="inlineStr">
         <is>
-          <t>交付完成</t>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B156" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B156" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B157" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B157" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B158" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46309</v>
+      </c>
+      <c r="B158" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B159" s="11" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B160" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46309</v>
+      </c>
+      <c r="B160" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B161" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46309</v>
+      </c>
+      <c r="B161" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="17" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
       <c r="B162" s="11" t="inlineStr">
         <is>
-          <t>复验通过</t>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B163" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46309</v>
+      </c>
+      <c r="B163" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B164" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+        <v>46309</v>
+      </c>
+      <c r="B164" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E164" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B165" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46309</v>
+      </c>
+      <c r="B165" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B166" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46309</v>
+      </c>
+      <c r="B166" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C166" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E166" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B167" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46309</v>
+      </c>
+      <c r="B167" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C167" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B168" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46309</v>
+      </c>
+      <c r="B168" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C168" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B169" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+        <v>46309</v>
+      </c>
+      <c r="B169" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C169" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D169" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -12713,24 +12713,24 @@
       <c r="A170" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B170" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B170" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C170" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -12738,24 +12738,24 @@
       <c r="A171" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B171" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B171" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C171" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D171" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -12763,24 +12763,24 @@
       <c r="A172" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B172" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B172" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C172" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -12795,17 +12795,17 @@
       </c>
       <c r="C173" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -12820,17 +12820,17 @@
       </c>
       <c r="C174" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E174" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -12838,19 +12838,19 @@
       <c r="A175" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B175" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B175" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C175" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
@@ -12863,20 +12863,24 @@
       <c r="A176" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B176" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C176" s="7" t="inlineStr"/>
+      <c r="B176" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C176" s="7" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E176" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -12884,20 +12888,24 @@
       <c r="A177" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B177" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
-        </is>
-      </c>
-      <c r="C177" s="7" t="inlineStr"/>
+      <c r="B177" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C177" s="7" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
       <c r="D177" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -12905,20 +12913,24 @@
       <c r="A178" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B178" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
-        </is>
-      </c>
-      <c r="C178" s="7" t="inlineStr"/>
+      <c r="B178" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C178" s="7" t="inlineStr">
+        <is>
+          <t>D5</t>
+        </is>
+      </c>
       <c r="D178" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12926,19 +12938,19 @@
       <c r="A179" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B179" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B179" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C179" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D179" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
@@ -12951,24 +12963,24 @@
       <c r="A180" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B180" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B180" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C180" s="7" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -12976,19 +12988,19 @@
       <c r="A181" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B181" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B181" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C181" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
@@ -13001,24 +13013,24 @@
       <c r="A182" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B182" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B182" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C182" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D182" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -13026,19 +13038,19 @@
       <c r="A183" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B183" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B183" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C183" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
@@ -13051,24 +13063,24 @@
       <c r="A184" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B184" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B184" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C184" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D184" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E184" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13083,17 +13095,17 @@
       </c>
       <c r="C185" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D185" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -13101,18 +13113,381 @@
       <c r="A186" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B186" s="19" t="inlineStr">
+      <c r="B186" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
+        </is>
+      </c>
+      <c r="C186" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="D186" s="7" t="inlineStr">
+        <is>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+        </is>
+      </c>
+      <c r="E186" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B187" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C186" s="7" t="inlineStr"/>
-      <c r="D186" s="7" t="inlineStr">
+      <c r="C187" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="D187" s="7" t="inlineStr">
+        <is>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+        </is>
+      </c>
+      <c r="E187" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 task/d13-boot fdbb217</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B188" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C188" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="D188" s="7" t="inlineStr">
+        <is>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+        </is>
+      </c>
+      <c r="E188" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B189" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
+        </is>
+      </c>
+      <c r="C189" s="7" t="inlineStr">
+        <is>
+          <t>D15</t>
+        </is>
+      </c>
+      <c r="D189" s="7" t="inlineStr">
+        <is>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+        </is>
+      </c>
+      <c r="E189" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 1995be8</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B190" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C190" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
+      <c r="D190" s="7" t="inlineStr">
+        <is>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+        </is>
+      </c>
+      <c r="E190" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B191" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C191" s="7" t="inlineStr"/>
+      <c r="D191" s="7" t="inlineStr">
+        <is>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+        </is>
+      </c>
+      <c r="E191" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B192" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C192" s="7" t="inlineStr"/>
+      <c r="D192" s="7" t="inlineStr">
+        <is>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+        </is>
+      </c>
+      <c r="E192" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B193" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C193" s="7" t="inlineStr"/>
+      <c r="D193" s="7" t="inlineStr">
+        <is>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+        </is>
+      </c>
+      <c r="E193" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B194" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C194" s="7" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="D194" s="7" t="inlineStr">
+        <is>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+        </is>
+      </c>
+      <c r="E194" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B195" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C195" s="7" t="inlineStr">
+        <is>
+          <t>D11</t>
+        </is>
+      </c>
+      <c r="D195" s="7" t="inlineStr">
+        <is>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+        </is>
+      </c>
+      <c r="E195" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B196" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C196" s="7" t="inlineStr">
+        <is>
+          <t>D12;D13;D14</t>
+        </is>
+      </c>
+      <c r="D196" s="7" t="inlineStr">
+        <is>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+        </is>
+      </c>
+      <c r="E196" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B197" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C197" s="7" t="inlineStr">
+        <is>
+          <t>D13</t>
+        </is>
+      </c>
+      <c r="D197" s="7" t="inlineStr">
+        <is>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+        </is>
+      </c>
+      <c r="E197" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B198" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C198" s="7" t="inlineStr">
+        <is>
+          <t>D15;D16</t>
+        </is>
+      </c>
+      <c r="D198" s="7" t="inlineStr">
+        <is>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+        </is>
+      </c>
+      <c r="E198" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B199" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
+        </is>
+      </c>
+      <c r="C199" s="7" t="inlineStr">
+        <is>
+          <t>KR5.2</t>
+        </is>
+      </c>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+        </is>
+      </c>
+      <c r="E199" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 49031f6</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B200" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C200" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D200" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E200" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B201" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
+        </is>
+      </c>
+      <c r="C201" s="7" t="inlineStr"/>
+      <c r="D201" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E186" s="7" t="inlineStr">
+      <c r="E201" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -17832,7 +18207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H70"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -17876,7 +18251,7 @@
         <v>46307</v>
       </c>
       <c r="B4" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C4" s="6" t="n">
         <v>5</v>
@@ -17890,7 +18265,7 @@
         <v>46308</v>
       </c>
       <c r="B5" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C5" s="6" t="n">
         <v>7</v>
@@ -17904,7 +18279,7 @@
         <v>46309</v>
       </c>
       <c r="B6" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C6" s="6" t="n">
         <v>8</v>
@@ -17918,7 +18293,7 @@
         <v>46310</v>
       </c>
       <c r="B7" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C7" s="6" t="n">
         <v>12</v>
@@ -17932,7 +18307,7 @@
         <v>46311</v>
       </c>
       <c r="B8" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C8" s="6" t="n">
         <v>20</v>
@@ -17946,7 +18321,7 @@
         <v>46312</v>
       </c>
       <c r="B9" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C9" s="6" t="n">
         <v>28</v>
@@ -17960,7 +18335,7 @@
         <v>46313</v>
       </c>
       <c r="B10" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>28</v>
@@ -17974,13 +18349,13 @@
         <v>46314</v>
       </c>
       <c r="B11" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C11" s="6" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
     </row>
     <row r="12">
@@ -17988,10 +18363,10 @@
         <v>46315</v>
       </c>
       <c r="B12" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D12" s="6" t="n"/>
     </row>
@@ -18000,10 +18375,10 @@
         <v>46316</v>
       </c>
       <c r="B13" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C13" s="6" t="n">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D13" s="6" t="n"/>
     </row>
@@ -18012,10 +18387,10 @@
         <v>46317</v>
       </c>
       <c r="B14" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D14" s="6" t="n"/>
     </row>
@@ -18024,10 +18399,10 @@
         <v>46318</v>
       </c>
       <c r="B15" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C15" s="6" t="n">
-        <v>38</v>
+        <v>44</v>
       </c>
       <c r="D15" s="6" t="n"/>
     </row>
@@ -18036,10 +18411,10 @@
         <v>46319</v>
       </c>
       <c r="B16" s="6" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="C16" s="6" t="n">
-        <v>42</v>
+        <v>49</v>
       </c>
       <c r="D16" s="6" t="n"/>
     </row>
@@ -19628,7 +20003,7 @@
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>方案合主线 be3b699 (uboot.env bootcmd 加 mmc rescan 重试 ×15); 待用户批准写卡 + 冷上电 20 次验收</t>
+          <t>方案 be3b699 已上 03 (uboot.env); 软重启 20/20 进内核; 冷上电 20 次等 USB 继电器 (LCUS-1) 到货自动跑</t>
         </is>
       </c>
     </row>
@@ -19732,15 +20107,17 @@
       <c r="E68" s="17" t="n">
         <v>46319</v>
       </c>
-      <c r="F68" s="17" t="n"/>
-      <c r="G68" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F68" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G68" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H68" s="7" t="inlineStr">
         <is>
-          <t>task/d33-jtag (agent)</t>
+          <t>dr1v90 23474c7 (复验 53/0, v1_bringup 96/0)</t>
         </is>
       </c>
     </row>
@@ -19768,15 +20145,17 @@
       <c r="E69" s="17" t="n">
         <v>46316</v>
       </c>
-      <c r="F69" s="17" t="n"/>
-      <c r="G69" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F69" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G69" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H69" s="7" t="inlineStr">
         <is>
-          <t>task/d34-v1odd (agent)</t>
+          <t>dr1v90 7253608 (复验 d25/d23/v1_bringup/d9 全过)</t>
         </is>
       </c>
     </row>
@@ -19804,15 +20183,281 @@
       <c r="E70" s="17" t="n">
         <v>46319</v>
       </c>
-      <c r="F70" s="17" t="n"/>
-      <c r="G70" s="15" t="inlineStr">
+      <c r="F70" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G70" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 ff1846a (regress 27/0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>D36</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>软件引脚/硬件假设对齐 10-15/16 投板版</t>
+        </is>
+      </c>
+      <c r="C71" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E71" s="17" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F71" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G71" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H71" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 f2584d9 (桥位流四套重出 0 违例)</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="inlineStr">
+        <is>
+          <t>D35</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>核实 V1 能否双面 (W6 光电冲突)</t>
+        </is>
+      </c>
+      <c r="C72" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D72" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E72" s="17" t="n">
+        <v>46316</v>
+      </c>
+      <c r="F72" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G72" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 2b111f0 (网表独立复核)</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>D37</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>主控 IO 1.8V 可行性 (用户定最终 2.5V)</t>
+        </is>
+      </c>
+      <c r="C73" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E73" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F73" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G73" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H73" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 f9ffbe9 d37_io18/REPORT.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="inlineStr">
+        <is>
+          <t>D38</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>V1 面 B 软件就绪 (IO 电压开关/面B RTL/桥B/JTAG 两器件/--faces AB)</t>
+        </is>
+      </c>
+      <c r="C74" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D74" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E74" s="17" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F74" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 ad201f9 (v1_bringup 110/0, 双面仿真 0 错)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>D39</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>SoC↔桥通信专项验证包 + PRBS 位流</t>
+        </is>
+      </c>
+      <c r="C75" s="6" t="inlineStr">
+        <is>
+          <t>2;4;7</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E75" s="17" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F75" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G75" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H75" s="7" t="inlineStr">
+        <is>
+          <t>dr1v90 3ef6b06 (85/0; e60cp 6d5b3db3, 主控 prbs e7c33e78)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="inlineStr">
+        <is>
+          <t>D40</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>双面主控位流编译通过 (TD hold 修复崩溃)</t>
+        </is>
+      </c>
+      <c r="C76" s="6" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D76" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E76" s="17" t="n">
+        <v>46319</v>
+      </c>
+      <c r="F76" s="17" t="n"/>
+      <c r="G76" s="15" t="inlineStr">
         <is>
           <t>🔄</t>
         </is>
       </c>
-      <c r="H70" s="7" t="inlineStr">
-        <is>
-          <t>task/v2-disp (agent)</t>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>task/d40-ab (agent)</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>V1-B1</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>V1 主控/桥位流按投板版出齐 (单面 io25 / PRBS / 面 B 桥)</t>
+        </is>
+      </c>
+      <c r="C77" s="6" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>公共</t>
+        </is>
+      </c>
+      <c r="E77" s="17" t="n">
+        <v>46317</v>
+      </c>
+      <c r="F77" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
+        </is>
+      </c>
+      <c r="H77" s="7" t="inlineStr">
+        <is>
+          <t>_work/v1_main_1019 (io25 2b4f3311, e60c 7f612855, e60cb f919ea30)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[D29] 03 冷上电 20/20 + 软重启 20/20 通过, D29 关闭; 日志 progress/d29_coldboot; 看板更新
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-19.xlsx
+++ b/docs/progress/显性目的进度_2026-10-19.xlsx
@@ -8565,7 +8565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J201"/>
+  <dimension ref="A1:J202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -8636,16 +8636,16 @@
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>0.9782608695652174</v>
+        <v>1</v>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>45/46</t>
+          <t>46/46</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>KR 25/25 + 交付 20/21 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
+          <t>KR 25/25 + 交付 21/21 — 统一口径：达成率_P = (P 目标已达标的 KR 数 + P 需要的交付里已完成数) ÷ (有 P 目标的 KR 数 + P 需要的交付总数)，P = V0 / V1 / V2。</t>
         </is>
       </c>
       <c r="G4" s="8" t="n">
@@ -8668,16 +8668,16 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>0.8529411764705882</v>
+        <v>0.8676470588235294</v>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>58/68</t>
+          <t>59/68</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>KR 17/24 + 交付 41/44 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
+          <t>KR 17/24 + 交付 42/44 — 只按「必须」项计：KR 全算必须；交付看 deliverables.csv 的「级别」列 (必须/加分)，加分项不进分子分母。</t>
         </is>
       </c>
       <c r="G5" s="8" t="n">
@@ -8700,16 +8700,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.7972972972972973</v>
+        <v>0.8108108108108109</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>59/74</t>
+          <t>60/74</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 15/24 + 交付 44/50 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 15/24 + 交付 45/50 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8821,13 +8821,13 @@
         <v>46314</v>
       </c>
       <c r="H11" s="9" t="n">
-        <v>0.9782999999999999</v>
+        <v>1</v>
       </c>
       <c r="I11" s="9" t="n">
-        <v>0.8529</v>
+        <v>0.8676</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.7973</v>
+        <v>0.8108</v>
       </c>
     </row>
     <row r="12">
@@ -10261,51 +10261,51 @@
     </row>
     <row r="72">
       <c r="A72" s="17" t="n">
-        <v>46313</v>
+        <v>46314</v>
       </c>
       <c r="B72" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
         <is>
-          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
+          <t>03 手动冷上电 20/20: 每次 U-Boot→读 env OK→boot.scr→进内核→login, 0 次停在 =&gt;, env 读失败 0 (u-boot 早期 -110 探测行仍有, 不影响); 加软重启 20/20, D29 关闭; USB 继电器不再需要</t>
         </is>
       </c>
       <c r="E72" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1017_03_24h</t>
+          <t>progress/d29_coldboot</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="17" t="n">
-        <v>46312</v>
-      </c>
-      <c r="B73" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46313</v>
+      </c>
+      <c r="B73" s="6" t="inlineStr">
+        <is>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
         <is>
-          <t>D27</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
+          <t>03 24 h 产品配置长跑 9/10 (主线 3bf094f, voxslice 63e7afea): 停摆 0/死 0, 完成率最低 100%, RSS 23.1 MB 不涨, 30/31 段推流正常; S5 FAIL = 03:00 WiFi 断 (gw 不回 ICMP, povnetd 60 s 后才重连, 两轮 wpa+dhcp, 155 s 恢复; PC 侧 No route to host 约 5 min), 第 6 段推流时长用完仍在重连 rc 2 → 开 D22b 把恢复压到 ≤30 s</t>
         </is>
       </c>
       <c r="E73" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/SPEC.md</t>
+          <t>progress/soak_v0/1017_03_24h</t>
         </is>
       </c>
     </row>
@@ -10313,24 +10313,24 @@
       <c r="A74" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B74" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B74" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
         <is>
-          <t>V2-5</t>
+          <t>D27</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
         <is>
-          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
+          <t>SoC↔桥边带全功能合主线 (复验含回归全过): 握手/闭环训练+自动重训/桥计数经 B2S 回传 povstat/S2B 桥寄存器读写/2260 表改写 ACK 回读/亮度黑场/看门狗 (修黑场死锁)/停转降亮/版本核对; 综合: 桥 e60c 167.33 MHz 0 违例 (余量 0.40%), 主控 UL_SB SWNS +0.002; 🔴 回板阻塞 SB_RSTN 被 R235 10k 下拉, 现役主控位流不驱动 → 用 D27 主控位流或 FPC63 临时上拉; 待定 H-1~H-4</t>
         </is>
       </c>
       <c r="E74" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_fmt/README.md</t>
+          <t>dr1v90 d27_link/SPEC.md</t>
         </is>
       </c>
     </row>
@@ -10345,17 +10345,17 @@
       </c>
       <c r="C75" s="7" t="inlineStr">
         <is>
-          <t>D28b</t>
+          <t>V2-5</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
+          <t>2 期主控字槽序格式器合主线 fb9e6eb (复验含回归全过): ul_fmt_p2 4 列乒乓 + LUT 重排, 真内容 40/12/60 片与 v2_ref 逐组 0 错, 反例全检出; SWNS +0.001 (hclk 真余量约 +0.30); POV_UL_GEOM=p2 改字槽序, 原列序档改名 p2c; 待: 桥 24 链 UL12 解包, 板端 --disp p2</t>
         </is>
       </c>
       <c r="E75" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/回板当天.md</t>
+          <t>dr1v90 v2_fmt/README.md</t>
         </is>
       </c>
     </row>
@@ -10363,24 +10363,24 @@
       <c r="A76" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B76" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B76" s="6" t="inlineStr">
+        <is>
+          <t>进展</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
         <is>
-          <t>D27b</t>
+          <t>D28b</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
         <is>
-          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
+          <t>回板脚本接 D27 合主线 (复验 78/0): 现役套 (023e6582+e60) 必须 FPC63 临时上拉 (脚本问答把关), D27 套 (主控 _sb.bin + 桥 e60c) 闭环训练; D27 套位流本体尚未出 → 开 D27b 出件</t>
         </is>
       </c>
       <c r="E76" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d27_link/README.md</t>
+          <t>dr1v90 v1_bringup/回板当天.md</t>
         </is>
       </c>
     </row>
@@ -10388,24 +10388,24 @@
       <c r="A77" s="17" t="n">
         <v>46312</v>
       </c>
-      <c r="B77" s="6" t="inlineStr">
-        <is>
-          <t>进展</t>
+      <c r="B77" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
         <is>
-          <t>V2-6</t>
+          <t>D27b</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
+          <t>D27 套回板位流出件合主线: 主控 pov_m90_pure_ul800_p1_b12_sb.bin a36365e9 (hclk +0.003 真余量约 +0.30, pclk200 +0.048 比现役 +0.006 宽), 桥 e60c e7289b13 (旧记 394cd71a 只差头部创建时间) / e60p8c bddcece3; 存 _work/d10_v1bit_out/ 与 gw5a_bridge/results/; 回板用 D27 套免 FPC63 飞线</t>
         </is>
       </c>
       <c r="E77" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 gw5a_bridge/p2/README.md</t>
+          <t>dr1v90 d27_link/README.md</t>
         </is>
       </c>
     </row>
@@ -10415,22 +10415,22 @@
       </c>
       <c r="B78" s="6" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
         <is>
-          <t>全套</t>
+          <t>V2-6</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
         <is>
-          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
+          <t>2 期桥合主线: p2 core 24 链 UL12 解包, BSRAM 37/56 (一颗 GW5A-25 够), Gowin 0 违例余量 +0.018 ns CLS 84%; 主控→桥→24×2260 端到端逐像素 0 错 (E1-E4, 反例 4/4); 预存窗口 15.3 rps 时仅 ±0.5 µs (上行占片周期 97.5%), 回板按实测重扫 START; 待硬件: UL_CLK 第 87 对放 3.3V bank, ACK 片外 3×8 选 1, 48 扫表 0x04 推导值; 顺修 D27 verify S 基线</t>
         </is>
       </c>
       <c r="E78" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ~/full_*.log</t>
+          <t>dr1v90 gw5a_bridge/p2/README.md</t>
         </is>
       </c>
     </row>
@@ -10440,22 +10440,22 @@
       </c>
       <c r="B79" s="6" t="inlineStr">
         <is>
-          <t>修复</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>全套</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
+          <t>最新主线 fdb63f4 全套 19 套: 15 过; v2_map G4 / v2_bridge S 为守护误报 (D27b 时序摘要) 已修 d4a4e3a; 🔴 d19 O4_fake / d20_smooth S2 真回归: 假转本地播放换网格率 = 1×转速 (半圈换未生效), 10-16 3cb39fc 时 d19 PASS → 疑 D20e --pl-gate, 已退回 D20e agent 查修</t>
         </is>
       </c>
       <c r="E79" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 slice/SPEC.md §13.2</t>
+          <t>dr1v90 ~/full_*.log</t>
         </is>
       </c>
     </row>
@@ -10465,22 +10465,22 @@
       </c>
       <c r="B80" s="6" t="inlineStr">
         <is>
-          <t>长跑</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
         <is>
-          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
+          <t>本地播放半圈换回归修复合主线 86caee5 (复验 d19 16/0, d20_smooth, d20d, d20e V1-V5 全过): 根因 2cd422a 对齐放行 (--pl-gate) 对本地帧也生效, 本地 15 fps+margin 0.9 时 m=2 压成 1×转速; 改为只作用推流帧; 02 开机演示配置 (10 fps/20/1.0) 推算不受影响; voxslice 新 md5 63e7afea, 下次部署换</t>
         </is>
       </c>
       <c r="E80" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/1016_wkend_24h</t>
+          <t>dr1v90 slice/SPEC.md §13.2</t>
         </is>
       </c>
     </row>
@@ -10490,7 +10490,7 @@
       </c>
       <c r="B81" s="6" t="inlineStr">
         <is>
-          <t>部署</t>
+          <t>长跑</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
@@ -10500,37 +10500,37 @@
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
+          <t>02 24 h 产品配置长跑 PASS 10/10 (主线 8eced5a, PLV=0 max-fps 20 margin 1.0): 停摆 0/死 0, 10 s 窗口完成率最低 100%, 最差小时未完成 0.0011%, 推流 29 段 rc 0 均 16.8 帧/s, 停推 32 次全 300 s 回本地, RSS 23.1→23.1 MB; 注: PC 侧 D 盘 EIO 致 soak.sh 末段退出 (板上照常跑满并自恢复, 日志手动取回判读), ping 只记前 46 次, push.txt 少 3 段</t>
         </is>
       </c>
       <c r="E81" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1017_*.log</t>
+          <t>progress/soak_v0/1016_wkend_24h</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="17" t="n">
-        <v>46311</v>
+        <v>46312</v>
       </c>
       <c r="B82" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>部署</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
+          <t>02/03 卡上 voxslice 换主线 86caee5 版 (63e7afea, 旧版留 .bak-0717), 重启验收: 03 6/6 PASS; 02 A5 首次 1243 帧/90 s (&lt;1260, 开机后 20 s 内推流) 其余全过, 随后连推 3 次 1351/1351/1349 帧 = 满 15 帧/s → 判为开机初期偶发</t>
         </is>
       </c>
       <c r="E82" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22c.board.log</t>
+          <t>progress/v0_accept/accept_1017_*.log</t>
         </is>
       </c>
     </row>
@@ -10538,9 +10538,9 @@
       <c r="A83" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B83" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B83" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
@@ -10550,12 +10550,12 @@
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
+          <t>上板故障演练 14/14 PASS (povnetd 1.2): 装后重启 88 s; 杀 sshd/mdns/povnetd 60/7/72 s; 杀 wpa ×3 12/32/22 s; 关网卡 ×3 22/32/34 s; 错 SSID→热点→自回 545 s; 看门狗复位 2 项 60/220 s 找回且记非正常结束。用户要求 '不插串口永远连得上' 达成; 合主线回归中</t>
         </is>
       </c>
       <c r="E83" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d22c.board.log</t>
         </is>
       </c>
     </row>
@@ -10563,24 +10563,24 @@
       <c r="A84" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B84" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B84" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
+          <t>不插串口永远连得上 合主线 (上板演练 14/14; 合并回归 D22/rotor_ops/D18/D13/live_push 全过, D13 补丁比较口径剔除 D22 块)。串口可永久拔</t>
         </is>
       </c>
       <c r="E84" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board5.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10588,9 +10588,9 @@
       <c r="A85" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B85" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B85" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
@@ -10600,12 +10600,12 @@
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
+          <t>上板 PASS: 假转 5→20→5 斜坡换档 2 次 + 强制轮换 6 次, 跨圈写 0, 超时 0, 对拍 2/0 与 12/0, 完成率 100%, 收尾回默认 0x20471019 (测试解析同 D19 修正)。合并分支 task/merge-d21 全回归 12 套进行中</t>
         </is>
       </c>
       <c r="E85" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_d21.board5.log</t>
         </is>
       </c>
     </row>
@@ -10620,12 +10620,12 @@
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
+          <t>每圈片数随转速换档合主线 (全回归 12 套通过; D18 V3 允许卡上默认 kit=D19 落后仓库 RTL=D21); 主线 voxslice 已修 sub01 隐患。下一步: V1 12-bit 位流按主线 (D19+D21+D8) 重综合</t>
         </is>
       </c>
       <c r="E86" s="7" t="inlineStr">
@@ -10638,9 +10638,9 @@
       <c r="A87" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B87" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B87" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
@@ -10650,12 +10650,12 @@
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
+          <t>内容帧率跟转速 voxlive --fps auto 合主线 d3f16f3 (默认不变; 主机空闲时离线复验 PASS, 之前失败为主机忙)。上板 A/B (583 rpm 固定 15 vs auto+板 20/1.0) 进行中</t>
         </is>
       </c>
       <c r="E87" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_A fps_B</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10663,9 +10663,9 @@
       <c r="A88" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B88" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B88" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C88" s="7" t="inlineStr">
@@ -10675,12 +10675,12 @@
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
+          <t>上板 A/B (假转 583 rpm, 无对拍, 逐帧): A 默认 (推 15 + 板 15/0.9) 14.85/s, 间隔 p50/p95 51.5/103 ms, 节拍偏差 p50/p95 23%/55%; B (推 auto + 板 max-fps 20 / margin 1.0) 19.14/s, 间隔 51.4/51.8 ms, 偏差 0%/1%, 最长 206 ms。B 明显更流畅; 测 C (转速取自板遥测) 后决定改开机默认</t>
         </is>
       </c>
       <c r="E88" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_C</t>
+          <t>soak_runs/fps_A fps_B</t>
         </is>
       </c>
     </row>
@@ -10688,24 +10688,24 @@
       <c r="A89" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B89" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B89" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
+          <t>测 C: 不手填转速时 auto 拿不到转速 → 退回 15 fps (povstat UDP 在 WSL NAT 收不到; 且 V0 2047 PL 位流遥测本无转速)。开 D20d: 推流 TCP ACK 扩展回传转速 (新旧兼容) + 默认改 板 max-fps 20/margin 1.0、推流 auto; 同时开 D10 V1 12-bit 位流按主线重综合</t>
         </is>
       </c>
       <c r="E89" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20d-ackrps db4ec93</t>
+          <t>soak_runs/fps_C</t>
         </is>
       </c>
     </row>
@@ -10720,17 +10720,17 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
+          <t>推流 ACK 扩展回传转速 (帧头 flags bit15 请求 → 板回 0x07+rps×100+max-fps+margin+半圈标志; 新旧三种组合逐字节兼容) + 默认 板 max-fps 20/margin 1.0、推流 --fps auto (不用手填): 离线假转 583 rpm 自动锁 19.49/s std 0.2 ms。复验 + 上板 D 组进行中</t>
         </is>
       </c>
       <c r="E90" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
+          <t>dr1v90 task/d20d-ackrps db4ec93</t>
         </is>
       </c>
     </row>
@@ -10740,22 +10740,22 @@
       </c>
       <c r="B91" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>D20d</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
+          <t>V1 主控 12-bit 位流按主线重综合 8 档时序全收住 (回板主用 ul800_p1_b12 md5 023e6582, 替换作废 df4f0bea); 修 D8 引入的 build.sh set -e 静默退出; 2 期 MAXMISS 系命令配错 (12-bit@800M 本就超片周期), 非回归; 回板步骤 BOARD_DAY.md。注: V1 线速 800M (派活单写 1.2G 是主会话笔误); 缺口: V1 真内容板端通路 (voxslice 只支持 2047 后端) 待立项</t>
         </is>
       </c>
       <c r="E91" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/fps_D</t>
+          <t>dr1v90 task/d10-v1bit 9a9acf8</t>
         </is>
       </c>
     </row>
@@ -10763,9 +10763,9 @@
       <c r="A92" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B92" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B92" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
@@ -10775,12 +10775,12 @@
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
+          <t>上板 D 组 (不手填任何参数): 推流经 ACK 扩展自动拿到转速并锁 19.4 帧/s ✅; 但间隔 p95 103 ms (&gt;5% 帧翻倍), 不如手填转速的 B 组 (p95 51.8) —— 估计转速与实际微差导致周期性滑格, 需相位锁定 (跟板端 ACK 节奏) 作后续。离线复验 (指定 BASE) PASS, 合主线回归中</t>
         </is>
       </c>
       <c r="E92" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>soak_runs/fps_D</t>
         </is>
       </c>
     </row>
@@ -10788,24 +10788,24 @@
       <c r="A93" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B93" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B93" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20d</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
+          <t>ACK 回传转速 + 默认推流 auto / 板 20/1.0 合主线 (合并回归 7 套通过)。卡上部署尚未更新 (下次装卡带上); 后续: 相位锁定消 5% 滑格</t>
         </is>
       </c>
       <c r="E93" s="7" t="inlineStr">
         <is>
-          <t>~/rv_deploy.board.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10813,24 +10813,24 @@
       <c r="A94" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B94" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B94" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>D10</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
+          <t>卡上部署更新到主线 1d23e50 (voxslice md5 ecdc246f = 主线, show_boot max-fps 20 / margin 1.0, QoS 0x0F, PL 0x20471019, D22 povreach); D19 上板假转扫点 PASS</t>
         </is>
       </c>
       <c r="E94" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>~/rv_deploy.board.log</t>
         </is>
       </c>
     </row>
@@ -10838,24 +10838,24 @@
       <c r="A95" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B95" s="6" t="inlineStr">
-        <is>
-          <t>验收</t>
+      <c r="B95" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D10</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
+          <t>V1 主控位流按主线重综合合主线 (复验 5/5: 构建记录/联合仿真/上行回归/MAXMISS 说明); 回板步骤 d10_v1bit/BOARD_DAY.md</t>
         </is>
       </c>
       <c r="E95" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10865,22 +10865,22 @@
       </c>
       <c r="B96" s="6" t="inlineStr">
         <is>
-          <t>开工</t>
+          <t>验收</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>D20e/D23</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
+          <t>用户重启板子后 V0 验收 6/6 PASS (不插串口): 按名字找回 / 守护进程齐 (voxslice povnetd povreach povmdns povstat) / 开机默认 PL+QoS 0x0F+位流 0x20471019 / WiFi -55 dBm ping 30 丢 0 / 推流 90 s 1339 帧=14.9 帧/s 对端关闭 / 推后 voxslice 不变。首跑遇 D 盘 EIO 中断后重跑; A5 判读正则修正</t>
         </is>
       </c>
       <c r="E96" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
+          <t>progress/v0_accept/</t>
         </is>
       </c>
     </row>
@@ -10888,24 +10888,24 @@
       <c r="A97" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B97" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B97" s="6" t="inlineStr">
+        <is>
+          <t>开工</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>D24</t>
+          <t>D20e/D23</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
+          <t>D20e 推流相位锁定 (消 auto 模式 5% 滑格) + D23 V1 真内容板端通路 并行开工; 用户新提: 开机默认动画要有立方体动图 (待做)</t>
         </is>
       </c>
       <c r="E97" s="7" t="inlineStr">
         <is>
-          <t>用户</t>
+          <t>dr1v90 task/d20e-phaselock task/d23-v1content</t>
         </is>
       </c>
     </row>
@@ -10913,24 +10913,24 @@
       <c r="A98" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B98" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B98" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>D23</t>
+          <t>D24</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
+          <t>用户: 开机动画就用现在这个 (geo_loop, 含线框立方体), 不换; D26 V2 位流构建放行, 主会话后台跑; 新板定名 DR1M90-03, 拷卡包 card_kit_dr1m90-03 待用户管理员运行 make_card.ps1</t>
         </is>
       </c>
       <c r="E98" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>用户</t>
         </is>
       </c>
     </row>
@@ -10945,12 +10945,12 @@
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>D20e</t>
+          <t>D23</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
+          <t>V1 显示后端 voxslice --disp 2260 合主线 a41d63b (独立复验 24/0, 合并后回归 d21/d23 过)</t>
         </is>
       </c>
       <c r="E99" s="7" t="inlineStr">
@@ -10963,24 +10963,24 @@
       <c r="A100" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B100" s="6" t="inlineStr">
-        <is>
-          <t>部署</t>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>D20e</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
+          <t>推流相位锁定合主线 c80f5fb: 583 rpm 滑格 5.2%→0.19%, 900 rpm 22%→0.12% (p95 = 理想间隔); 代价 延迟 120→170-250 ms (--phaselock off 可回老行为)</t>
         </is>
       </c>
       <c r="E100" s="7" t="inlineStr">
         <is>
-          <t>progress/v0_accept/accept_1016_d20e.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -10988,24 +10988,24 @@
       <c r="A101" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B101" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B101" s="6" t="inlineStr">
+        <is>
+          <t>部署</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>KR7.3/D24</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
+          <t>02 卡上 voxslice 换 D20e 版 (ba243d71, 旧版留 .bak-d20e), 重启后 V0 验收 6/6 PASS (推流 1326 帧/90 s, WiFi -44 dBm 丢 0)</t>
         </is>
       </c>
       <c r="E101" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>progress/v0_accept/accept_1016_d20e.log</t>
         </is>
       </c>
     </row>
@@ -11013,24 +11013,24 @@
       <c r="A102" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B102" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B102" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>KR7.3/D24</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
+          <t>KR7.3 16 位计数回绕修正合主线 (存档无原始计数, 99.84% 无法重算; 38/57 转动行待核); D24 立方体候选合主线, 用户定开机保持 geo_loop</t>
         </is>
       </c>
       <c r="E102" s="7" t="inlineStr">
         <is>
-          <t>D:\card03</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11038,24 +11038,24 @@
       <c r="A103" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B103" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B103" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>D25</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
+          <t>第二块板: 公司 DLP 拦 TF 卡文件写入 → WSL 做 512 MB 镜像 + host/flash_card_raw.ps1 块级写, 读回 PASS; 等上电按名字找</t>
         </is>
       </c>
       <c r="E103" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>D:\card03</t>
         </is>
       </c>
     </row>
@@ -11063,24 +11063,24 @@
       <c r="A104" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B104" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B104" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D25</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
+          <t>V1 换档合主线 90b1d79: 358/286/210 档 (阈值 11.6/14.6 rps, 回差), 各档最高转速桥余量 3.9/3.3/2.7%; 不改 RTL 不重出位流; 顺修 --local-always SIGTERM 挂死; 卡上 voxslice 仍 D20e 版 (V0 dump 逐字节同, 不急换)</t>
         </is>
       </c>
       <c r="E104" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\cap_COM29.log</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11095,17 +11095,17 @@
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>回归</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
+          <t>用户改供电上电后: mDNS 查不到, 串口 COM29/COM30 (CH342) 140 s 无输出、回车无回显; 后台录串口 2 h + 寻板 3 h; 待用户回来断电重上电</t>
         </is>
       </c>
       <c r="E105" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20d_ackrps d20c_fps</t>
+          <t>D:\card03\cap_COM29.log</t>
         </is>
       </c>
     </row>
@@ -11113,24 +11113,24 @@
       <c r="A106" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B106" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>回归</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
+          <t>d20d P2 / d20c F3 帧间隔 std 判据在机器高负载 (load 4-6, D25 全量 + D26 TD) 时偶发超门槛 (4.6/8.3 ms vs &lt;4), 空闲同代码 0.1 ms; 待空闲复测, 必要时改失败重测一次</t>
         </is>
       </c>
       <c r="E106" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d12_latency/RESULTS.md</t>
+          <t>dr1v90 d20d_ackrps d20c_fps</t>
         </is>
       </c>
     </row>
@@ -11145,17 +11145,17 @@
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>D9</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
+          <t>延迟复测合主线: 相位锁定 auto 保持, lock-lead 150→70 ms; 583 rpm 延迟 p50/p95/p99 133/138/155 ms (锁相关 126/127/196, 滑格 2.1%→0.14%); 900 rpm 122/206/276 ms 滑格 0.37%; 帧间隔 p95 = 理想</t>
         </is>
       </c>
       <c r="E107" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d9_e2e/</t>
+          <t>dr1v90 d12_latency/RESULTS.md</t>
         </is>
       </c>
     </row>
@@ -11163,24 +11163,24 @@
       <c r="A108" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B108" s="6" t="inlineStr">
-        <is>
-          <t>硬件</t>
+      <c r="B108" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>DR1M90-03</t>
+          <t>D9</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
+          <t>V1 端到端仿真合主线: 真内容主机→板端→主控 RTL→上行→桥→6×2260 模型, 逐像素 0 错; 反例 3/3; 358 档只跑回绕窗口 (整圈用 N=16), 只 12-bit/假角度</t>
         </is>
       </c>
       <c r="E108" s="7" t="inlineStr">
         <is>
-          <t>D:\card03\boot03.log</t>
+          <t>dr1v90 d9_e2e/</t>
         </is>
       </c>
     </row>
@@ -11188,24 +11188,24 @@
       <c r="A109" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B109" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B109" s="6" t="inlineStr">
+        <is>
+          <t>硬件</t>
         </is>
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>D26</t>
+          <t>DR1M90-03</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
+          <t>03 起来了: 控制台 COM30 (CH342-A); 冷上电 u-boot 报 Card did not respond to voltage select -110 停在 =&gt;, mmc rescan + boot 后正常; 登记 dr1m90-03 (10.10.21.10), V0 验收 6/6 PASS (WiFi -45 dBm, 推流 1351 帧/90 s) → D29 查根因</t>
         </is>
       </c>
       <c r="E109" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
+          <t>D:\card03\boot03.log</t>
         </is>
       </c>
     </row>
@@ -11213,24 +11213,24 @@
       <c r="A110" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B110" s="6" t="inlineStr">
-        <is>
-          <t>开工</t>
+      <c r="B110" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>周末</t>
+          <t>D26</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
+          <t>V2 位流按主线重出合主线 c8e8294: 0 违例但余量 0.000 ns (旧 +0.001), 资源略降; D26 agent 遗留的卡死构建进程 (嵌套 flock) 占锁 2.5 h, 已按 PID 清掉</t>
         </is>
       </c>
       <c r="E110" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
+          <t>dr1v90 td_pov/pure_ul/results/p2_ul1200_b12_v3</t>
         </is>
       </c>
     </row>
@@ -11240,22 +11240,22 @@
       </c>
       <c r="B111" s="6" t="inlineStr">
         <is>
-          <t>方案</t>
+          <t>开工</t>
         </is>
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>D29</t>
+          <t>周末</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
+          <t>用户: SoC↔桥通信全功能开工, 软件能做的都做, 周一看结果。开 D27 (SoC↔桥全功能, Opus) / D28 (V1 回板一键脚本) / D29 (冷启动认卡); 02 跑 24 h 产品配置长跑 (PLV=0 max-fps 20 margin 1.0, 主线 8eced5a)</t>
         </is>
       </c>
       <c r="E111" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d29_sdboot/PLAN.md</t>
+          <t>dr1v90 soak8h/runs/1016_wkend_24h</t>
         </is>
       </c>
     </row>
@@ -11263,24 +11263,24 @@
       <c r="A112" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B112" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B112" s="6" t="inlineStr">
+        <is>
+          <t>方案</t>
         </is>
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>D28</t>
+          <t>D29</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
+          <t>03 冷启动认卡: 热重启 13/13 无法复现, 最可能 u-boot sdhci 首次 mmc_init 间歇失败且 an_bootcmd 无重试; 方案 A 只改卡上 uboot.env 的 bootcmd (mmc rescan 重试 15 次, 其余 49 变量逐字节同, md5 dae13f64), u-boot 提示符手敲已验证; 等用户批准写卡 + 冷上电 20 次验收 (判据 20/20); 发现 03 未装 S00sdoff 钩子</t>
         </is>
       </c>
       <c r="E112" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v1_bringup/</t>
+          <t>dr1v90 d29_sdboot/PLAN.md</t>
         </is>
       </c>
     </row>
@@ -11288,24 +11288,24 @@
       <c r="A113" s="17" t="n">
         <v>46311</v>
       </c>
-      <c r="B113" s="6" t="inlineStr">
-        <is>
-          <t>修复</t>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>D30</t>
+          <t>D28</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
+          <t>V1 回板一键脚本合主线: bringup.sh S0 前置 → S9 恢复, 每步 CHECK + 失败原因/下一步; 演练 (假寄存器/qemu) 74 PASS, 12 种故障注入全命中; 待真板核: 位流加载/真线速误码/真画面/桥 UART 字符串</t>
         </is>
       </c>
       <c r="E113" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
+          <t>dr1v90 v1_bringup/</t>
         </is>
       </c>
     </row>
@@ -11315,22 +11315,22 @@
       </c>
       <c r="B114" s="6" t="inlineStr">
         <is>
-          <t>进展</t>
+          <t>修复</t>
         </is>
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>V2-3</t>
+          <t>D30</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
+          <t>回归计时判据 (d20d P2 / d20c F3) 抗机器忙合主线: 稳健 std + 失败重测; load 17-31 下 5/5 PASS, 反例全检出</t>
         </is>
       </c>
       <c r="E114" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 v2_map/DESIGN.md</t>
+          <t>dr1v90 d20c_fps/test_d30_judge.sh</t>
         </is>
       </c>
     </row>
@@ -11340,47 +11340,47 @@
       </c>
       <c r="B115" s="6" t="inlineStr">
         <is>
-          <t>评估</t>
+          <t>进展</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>D31</t>
+          <t>V2-3</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
+          <t>2 期 192×216 映射离线完成合主线 691a772 (复验 15/15): p2_192x216 profile, 605 档 == 生产表, v2_ref.py/disp_p2.c 与 2 期全链 tb 逐组对拍; 发现 2 期上行 (105.33 µs/片) 比 2260 更紧, 605/512 两档只到 1110 rpm → 建议 605/513/461; 主控缺列序→字槽序格式器 (方案已证); 9 项待硬件确认 (H1-H9); 待用户定档表</t>
         </is>
       </c>
       <c r="E115" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 d31_v1odd/REPORT.md</t>
+          <t>dr1v90 v2_map/DESIGN.md</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="17" t="n">
-        <v>46310</v>
-      </c>
-      <c r="B116" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46311</v>
+      </c>
+      <c r="B116" s="6" t="inlineStr">
+        <is>
+          <t>评估</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D31</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
+          <t>V1 偶数片数漏柱: 面 A 过转轴, 偶数后半圈与前半圈取样重合; 两面漏柱 358/286/210 = 124/458/1524 → 357/285/209 = 0/62/467; 只改档表不动 RTL, 桥余量略宽; 另: D25 阈值下 12 rps 落在 286 档; 待用户定</t>
         </is>
       </c>
       <c r="E116" s="7" t="inlineStr">
         <is>
-          <t>progress/soak_v0/report.md</t>
+          <t>dr1v90 d31_v1odd/REPORT.md</t>
         </is>
       </c>
     </row>
@@ -11388,24 +11388,24 @@
       <c r="A117" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B117" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>QoS</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
+          <t>8 h 无人值守长跑 9/9 通过 (重开轮 23:45-07:45; 判读 S1 行数口径误判已改为覆盖时长 fe53bde); V0 出口 ⑥ 达成 → V0 出口 8/8</t>
         </is>
       </c>
       <c r="E117" s="7" t="inlineStr">
         <is>
-          <t>~/qos_runs</t>
+          <t>progress/soak_v0/report.md</t>
         </is>
       </c>
     </row>
@@ -11420,17 +11420,17 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>D16b</t>
+          <t>QoS</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
+          <t>QoS (XMON DDR_S2 QOS_CONFIG=0x0F) 带载对照 (纯切片 30 Hz): 体素流+TCP 迟到 4.12% → 0.000%, CPU memcpy 300 MB/s 91.5% → 0.000%; 2047 32 bit@16.15 rps 完成率无改善 (86/71% vs 无 QoS 91/82%, 带宽上限); 测后寄存器已写回 0</t>
         </is>
       </c>
       <c r="E118" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16b-tile 7936b7e</t>
+          <t>~/qos_runs</t>
         </is>
       </c>
     </row>
@@ -11438,24 +11438,24 @@
       <c r="A119" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B119" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B119" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D16b</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
+          <t>4x4 分块上板 A/B: 体素流+TCP 迟到 现布局 5.34%/4.45% (漂移 0.89 pp) vs 分块 4.79%, 收益在漂移内 = 无效; 迟到角度随相位漂移, 非几何换行主导。按约定不合主线, 分支 task/d16b-tile 保留</t>
         </is>
       </c>
       <c r="E119" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>dr1v90 task/d16b-tile 7936b7e</t>
         </is>
       </c>
     </row>
@@ -11470,12 +11470,12 @@
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
+          <t>用户定 V0/V1/V2 兼容 300-1200 rpm; 实转 583 rpm PL 只 8 fps (等整圈换帧) → D19 半圈换帧开做 (RTL+voxslice+假转扫速验收)</t>
         </is>
       </c>
       <c r="E120" s="7" t="inlineStr">
@@ -11488,24 +11488,24 @@
       <c r="A121" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B121" s="6" t="inlineStr">
-        <is>
-          <t>分析</t>
+      <c r="B121" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>V1/V2</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
+          <t>用户定流畅显示为一等要求 (V0/V1/V2); D20 阶段 1 流畅度指标+门槛+基线开做 (与 D19 并行)</t>
         </is>
       </c>
       <c r="E121" s="7" t="inlineStr">
         <is>
-          <t>budget/rpm_range_2026-10-15.md</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11513,24 +11513,24 @@
       <c r="A122" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B122" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B122" s="6" t="inlineStr">
+        <is>
+          <t>分析</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>KR7.3</t>
+          <t>V1/V2</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
+          <t>转速 300-1200 rpm 纸面预算: 300 rpm 体刷新仅 10 Hz (物理闪烁); V1 358 片只到 ~718 rpm, 1200 需降到 215 片; V2 605 片到 ~1060 rpm; 公共切片核需支持运行时换每圈片数 (见 budget/rpm_range_2026-10-15.md)</t>
         </is>
       </c>
       <c r="E122" s="7" t="inlineStr">
         <is>
-          <t>progress/realspin_v0/</t>
+          <t>budget/rpm_range_2026-10-15.md</t>
         </is>
       </c>
     </row>
@@ -11538,19 +11538,19 @@
       <c r="A123" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B123" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>KR7.3</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
+          <t>实转 1 h 无故障通过 (583 rpm, QoS 开机默认已上卡 7d301a6); V0 必须项全部达成</t>
         </is>
       </c>
       <c r="E123" s="7" t="inlineStr">
@@ -11563,24 +11563,24 @@
       <c r="A124" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B124" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
+          <t>实转换帧仅 10.45/s (583 rpm 整圈换帧限制), 用户感觉卡; D19 半圈换帧 + D20 流畅度门槛处理</t>
         </is>
       </c>
       <c r="E124" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20-smooth 83a5fd7</t>
+          <t>progress/realspin_v0/</t>
         </is>
       </c>
     </row>
@@ -11588,24 +11588,24 @@
       <c r="A125" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B125" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B125" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D20</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
+          <t>流畅度阶段 1: host/smooth_report.py + 门槛 (软件损失≤3%, 间隔 p99≤2T0, 长停顿≤5‰, 撕裂 0 等, SPEC §12) + voxslice --flip-log; 基线: 8 h 假转软件损失 2.3% 但约每 2 min 一次 2-3 s 无新帧 (主机/链路侧, 板端 PL 无缺口) 判 FAIL; 实转 648 rpm 软件损失 3.5%, 每分钟至少一顿 0.3-1.1 s 判 FAIL。主会话复验中</t>
         </is>
       </c>
       <c r="E125" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 e215176</t>
+          <t>dr1v90 task/d20-smooth 83a5fd7</t>
         </is>
       </c>
     </row>
@@ -11613,24 +11613,24 @@
       <c r="A126" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B126" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
+          <t>更多内容 + 手机网页控制合主线 (用户实转看过); 新克隆回归全过</t>
         </is>
       </c>
       <c r="E126" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d19-halfrev 1beafa6</t>
+          <t>dr1v90 e215176</t>
         </is>
       </c>
     </row>
@@ -11645,17 +11645,17 @@
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>D20b</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
+          <t>半圈换帧: 换网格上限 1×→2×转速 (583 rpm 9.7→~19/s), 慢转均匀丢帧; 16/32 档位流时序收住 (REV 0x20471019/1A); 转速窗口 300-1200; 离线 16/16 + 仿真 21+5 + pls2047 32/32。主会话复验+上板假转扫点中</t>
         </is>
       </c>
       <c r="E127" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20b-sim 9081f62</t>
+          <t>dr1v90 task/d19-halfrev 1beafa6</t>
         </is>
       </c>
     </row>
@@ -11665,22 +11665,22 @@
       </c>
       <c r="B128" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>D19</t>
+          <t>D20b</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
+          <t>画面模拟器 host/pov_view.py (按视觉暂留合成人眼所见, 并排对比): 整圈换帧 9.8/s 跳 51 帧; 半圈 15/s 但 51/103 ms 交替 (内容 15 fps 与半圈节拍不齐 → D20 阶段 3 内容帧率跟转速); 300 rpm 闪烁; 停推冻结后跳帧。示例 gif 在 dr1v90/_work/d20b/d20_smooth/sim_out/; 复验 PASS</t>
         </is>
       </c>
       <c r="E128" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/merge-d19-d20 106364e</t>
+          <t>dr1v90 task/d20b-sim 9081f62</t>
         </is>
       </c>
     </row>
@@ -11688,24 +11688,24 @@
       <c r="A129" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B129" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B129" s="6" t="inlineStr">
+        <is>
+          <t>验证</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>D19/D20</t>
+          <t>D19</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
+          <t>半圈换帧上板假转扫点 PASS: 5/7.5/10/15/20 rps 换网格 9.00/13.56/15.09/15.09/15.08 每秒 (老行为 10 rps 仅 9.00), 完成率 100%, 撕裂 0, 对拍全一致, 超时 0; 卡上开机默认已是 D19 位流 0x20471019。D19+D20+D20b 合并分支全回归中</t>
         </is>
       </c>
       <c r="E129" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/merge-d19-d20 106364e</t>
         </is>
       </c>
     </row>
@@ -11713,24 +11713,24 @@
       <c r="A130" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B130" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B130" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D19/D20</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
+          <t>半圈换帧 + 流畅度检测 + 画面模拟器合主线; 全回归 10 套 (D18/D13/D19/D20/D20b/color/pls2047/rotor_ops/live_push/重连) 通过; 下一步 D20 阶段 3 (内容帧率跟转速、主机侧停顿诊断) + 实转复核</t>
         </is>
       </c>
       <c r="E130" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband adeba44</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11740,22 +11740,22 @@
       </c>
       <c r="B131" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>D20/D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
+          <t>每圈片数随转速换档 (V1/V2 到 1200 rpm 的前提): N/PB/LUT 圈边界同步锁存, 回差 5%; V0 2047 人为 142/128 两档仿真逐字节一致、撕裂 0, 假转斜坡升降各 1 次不抖; 16/32 档位流时序收住 (REV 0x20471021/22)。风险: 软件写序时间窗 (可加影子寄存器)。主会话复验中, 诊断跑完后上板</t>
         </is>
       </c>
       <c r="E131" s="7" t="inlineStr">
         <is>
-          <t>~/realspin/tcp</t>
+          <t>dr1v90 task/d21-nband adeba44</t>
         </is>
       </c>
     </row>
@@ -11763,24 +11763,24 @@
       <c r="A132" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B132" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B132" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D20/D22</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
+          <t>推流每 124.5 s 卡 3 s 的根因 = 长跑脚本的板上对拍 (--pl-verify 1800 ≈ 每 120 s, 每次停 ~3 s), 测试工具自身, 产品默认不开; WiFi 链路同刻 ping 0 丢。WSL/Windows 各 6 min 回放对照: 无周期卡顿, 但有偶发 1-1.7 s ACK 停顿 (每 6 min 1-2 次) = 真实 WiFi 抖动 → D22 WiFi 稳定 (用户 10-15: V0 必须搞定, 不能靠串口)</t>
         </is>
       </c>
       <c r="E132" s="7" t="inlineStr">
         <is>
-          <t>用户 10-15</t>
+          <t>~/realspin/tcp</t>
         </is>
       </c>
     </row>
@@ -11788,9 +11788,9 @@
       <c r="A133" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B133" s="6" t="inlineStr">
-        <is>
-          <t>交付</t>
+      <c r="B133" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
@@ -11800,12 +11800,12 @@
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
+          <t>用户: 不插串口也必须永远连得上, 彻底解决 (V0 必须) → D22 四层兜底开做: 服务监护 + 硬件看门狗 + 兜底热点 + 故障注入验收</t>
         </is>
       </c>
       <c r="E133" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach ee4a55c</t>
+          <t>用户 10-15</t>
         </is>
       </c>
     </row>
@@ -11820,17 +11820,17 @@
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>D20c</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
+          <t>不插串口永远连得上: povreach 服务监护 + 硬件看门狗 (60 s, 防风暴) + 兜底热点 POV-&lt;板名&gt; (hostapd 静编, 192.168.77.1, 状态页可填 WiFi) + 30 min 无网重启; 失效模式表 16 行; 离线 9/9。排队上板故障演练 (8 项, 含 2 次看门狗复位)</t>
         </is>
       </c>
       <c r="E134" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d20c-fps 338eaaf</t>
+          <t>dr1v90 task/d22-reach ee4a55c</t>
         </is>
       </c>
     </row>
@@ -11840,7 +11840,7 @@
       </c>
       <c r="B135" s="6" t="inlineStr">
         <is>
-          <t>复验</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
@@ -11850,12 +11850,12 @@
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
+          <t>内容帧率跟转速 voxlive --fps auto: 583 rpm 换帧间隔 std 23.4→0.1-0.9 ms (离线假转)。取舍: 板端默认 (max-fps 15, margin 0.9) 下 583 rpm 均匀但仅 9.7 fps; 板端 max-fps 20 + margin 1.0 → 19.4 fps 均匀。计划 D22 后上板验证 20/1.0 后改开机默认</t>
         </is>
       </c>
       <c r="E135" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d20c.v.log</t>
+          <t>dr1v90 task/d20c-fps 338eaaf</t>
         </is>
       </c>
     </row>
@@ -11865,22 +11865,22 @@
       </c>
       <c r="B136" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>复验</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>D8</t>
+          <t>D20c</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
+          <t>复验 F3 端到端节拍均匀度在主机忙 (D8 大仿真并行) 时不达标: 583 auto std 9.0/5.2 ms (门槛 3/4), 帧率正确; 主机计时抖动敏感, 先不合主线, 待空闲复验 + 上板实测定</t>
         </is>
       </c>
       <c r="E136" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d8-cosim 85dfe51</t>
+          <t>~/rv_d20c.v.log</t>
         </is>
       </c>
     </row>
@@ -11888,9 +11888,9 @@
       <c r="A137" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B137" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B137" s="6" t="inlineStr">
+        <is>
+          <t>交付</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
@@ -11900,12 +11900,12 @@
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
+          <t>V1 主控↔桥↔2260 联合仿真 0 错 (12/8 bit, 6 链×16 片, 训练锁定, 半圈换帧); 抓出并修 2 个回板必错 bug: 12-bit 字槽格式主控两 beat vs 桥紧排不一致 (改主控 PK12, 上行 195→110 µs/片) + 1 期切片器 NXG 未传 (160 宽按 192 算); 待: 1 期 12-bit 位流重综合 (hclk 余量原 +0.001 ns)</t>
         </is>
       </c>
       <c r="E137" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 feature/lvds-b2b</t>
+          <t>dr1v90 task/d8-cosim 85dfe51</t>
         </is>
       </c>
     </row>
@@ -11913,24 +11913,24 @@
       <c r="A138" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B138" s="6" t="inlineStr">
-        <is>
-          <t>测量</t>
+      <c r="B138" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>D22/D20</t>
+          <t>D8</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
+          <t>V1 联合仿真合主线 (新克隆复验 5/5; 合并回归 sim_v1/pls2047/D18/D19 通过, D19 O4 一次主机忙计时抖动重跑过); V1 回板就绪清单 ⑤ 达成</t>
         </is>
       </c>
       <c r="E138" s="7" t="inlineStr">
         <is>
-          <t>soak_runs/netdiag_1015_1814</t>
+          <t>dr1v90 feature/lvds-b2b</t>
         </is>
       </c>
     </row>
@@ -11938,24 +11938,24 @@
       <c r="A139" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B139" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B139" s="6" t="inlineStr">
+        <is>
+          <t>测量</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22/D20</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
+          <t>1 h 产品配置 (无对拍) 推流诊断: 换帧 14.64/s 软件损失 2.4% ✅, 间隔 p99 124 ms ✅, 长停顿 3.7‰ ✅, 最长 495 ms ❌ (门槛 267); PC→板 ping 16781/0 丢; &gt;0.5 s ACK 停顿 46 min 内 4 次 (最长 0.78 s), 同刻 PC→网关 RTT 165-275 ms = PC 侧 WiFi 抖动。周期 3 s 卡顿消失 (确认系对拍)。余项: 0.5-0.8 s 偶发抖动 (播放缓冲 vs 延迟取舍 / PC 有线或专用路由)</t>
         </is>
       </c>
       <c r="E139" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d21.board.log</t>
+          <t>soak_runs/netdiag_1015_1814</t>
         </is>
       </c>
     </row>
@@ -11970,17 +11970,17 @@
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
+          <t>换档位流 (REV 0x20471021) 上板起步即停摆 (档 0 未换档时写完 47 片后停, 换网格全超时), 仿真全过 → 硅上与仿真不同; D21b 开查根因。另: D21 上板收尾用 m90/up.sh 会让板子没 PL, 已重启回开机默认 (0x20471019 + QoS)</t>
         </is>
       </c>
       <c r="E140" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach</t>
+          <t>~/rv_d21.board.log</t>
         </is>
       </c>
     </row>
@@ -12000,7 +12000,7 @@
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
+          <t>新克隆离线 O6 误 FAIL: hostapd/povreach 二进制 git 模式 644, WSL 本地盘克隆不可执行, qemu 静默拒绝 (板上 autorun 有 chmod, 不受影响); 已修 (git +x, verify chmod), 重跑后自动上板演练</t>
         </is>
       </c>
       <c r="E141" s="7" t="inlineStr">
@@ -12013,9 +12013,9 @@
       <c r="A142" s="17" t="n">
         <v>46310</v>
       </c>
-      <c r="B142" s="6" t="inlineStr">
-        <is>
-          <t>验证</t>
+      <c r="B142" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
@@ -12025,12 +12025,12 @@
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
+          <t>首轮上板演练 9 项误 FAIL = 验收脚本 info() 把板上 board_d22.sh info 的非 0 退出码当失败 (内容正常), settle/wait_healthy 恒失败; 板子本身正常 (装好开机 healthy, povreach managed, 看门狗 armed)。已修, 单独重跑全套演练 (~80 min); 期间 D21 取证因同时上板被干扰, 待 D22 后单独跑</t>
         </is>
       </c>
       <c r="E142" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22.board2.log</t>
+          <t>dr1v90 task/d22-reach</t>
         </is>
       </c>
     </row>
@@ -12040,22 +12040,22 @@
       </c>
       <c r="B143" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
+          <t>第二轮上板演练 (单独): 杀 sshd/mdns/povnetd 27-72 s 自愈找回 ✅; 错 SSID → 兜底热点 → 自己回公司网 ✅ (但 23.5 min, 目标 ≤10); 杀 wpa/关网卡、装后重启: 板子恢复了但 mDNS 按名字 240 s 内找不回 ❌ (缓存 IP 可连); 看门狗复位发生但晚于测试判定、卡上未记非正常结束 ❌。交回 D22 agent 修 (mDNS 找回为主)</t>
         </is>
       </c>
       <c r="E143" s="7" t="inlineStr">
         <is>
-          <t>~/d21b_forensic.log</t>
+          <t>~/rv_d22.board2.log</t>
         </is>
       </c>
     </row>
@@ -12070,17 +12070,17 @@
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>D22</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
+          <t>板上取证: 显示每圈取满 142 片, 但 s3rt_sys 旁听只认片号 0..47 → PL 每圈 48 触发后停摆; 不带档位 / 补 sub10 都一样 → RTL 旁听上限 (D21 改为按 FBO) 问题。交回 D21b 修 RTL; 板子已重启回默认 0x20471019</t>
         </is>
       </c>
       <c r="E144" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach 0d1da09</t>
+          <t>~/d21b_forensic.log</t>
         </is>
       </c>
     </row>
@@ -12090,7 +12090,7 @@
       </c>
       <c r="B145" s="6" t="inlineStr">
         <is>
-          <t>验证</t>
+          <t>根因</t>
         </is>
       </c>
       <c r="C145" s="7" t="inlineStr">
@@ -12100,12 +12100,12 @@
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
+          <t>按名字找不回的根因: povmdns 在地址回来/重关联时不重新发 IGMP 报告 (重复入组 EADDRINUSE 无报告), 企业 AP 只把组播转给报告过的站点 → mDNS 查询数分钟到不了板。修: 重关联/地址变化时退组再入组 + 宣告 (0/1/3/7/15/30 s) + 每 60 s 刷新; 看门狗读回实际超时并减半到 ≤60 s; 卡上记非正常结束。离线 10/10, 上板复验中</t>
         </is>
       </c>
       <c r="E145" s="7" t="inlineStr">
         <is>
-          <t>~/rv_d22b.board.log</t>
+          <t>dr1v90 task/d22-reach 0d1da09</t>
         </is>
       </c>
     </row>
@@ -12115,7 +12115,7 @@
       </c>
       <c r="B146" s="6" t="inlineStr">
         <is>
-          <t>交付</t>
+          <t>验证</t>
         </is>
       </c>
       <c r="C146" s="7" t="inlineStr">
@@ -12125,12 +12125,12 @@
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
+          <t>第三轮上板演练 9/10: 装后重启 24 s 按名字找回 ✅ (上轮找不回); sshd/mdns/povnetd 杀掉 38-72 s ✅; 关网卡 191 s ✅; 错 SSID→热点→自动回 543 s ✅ (上轮 1411); 看门狗复位 reachkill 54 s / netdstop 213 s 且记非正常结束 ✅ (实际超时 32 s); 仅 kill wpa_supplicant 240 s 内未找回 ❌ (随后恢复), 单独重跑定位中</t>
         </is>
       </c>
       <c r="E146" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d22-reach e438a12</t>
+          <t>~/rv_d22b.board.log</t>
         </is>
       </c>
     </row>
@@ -12140,47 +12140,47 @@
       </c>
       <c r="B147" s="6" t="inlineStr">
         <is>
-          <t>根因</t>
+          <t>交付</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>D21</t>
+          <t>D22</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
+          <t>povnetd 1.2: wpa 进程没了/卡死/接口 down 立即重连 (原来一律等 60 s, 且 60 s 后的重连反把已自愈的连接打断 → 73-240+ s 且不稳); 只丢包仍按 60 s 防误重连; 关键事件写卡 (复位后可查); verify wpakill/ifdown 各连跑 3 次、120 s 内按名字找回。离线 11/11, 上板全套复验中</t>
         </is>
       </c>
       <c r="E147" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d21-nband 084bba3</t>
+          <t>dr1v90 task/d22-reach e438a12</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="17" t="n">
-        <v>46309</v>
-      </c>
-      <c r="B148" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+        <v>46310</v>
+      </c>
+      <c r="B148" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>D3</t>
+          <t>D21</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>上行出口全量复验 45/0, 合主线</t>
+          <t>停摆根因不在 RTL: voxslice --pl 从不写显示 0x0C sub01 (bpp3), 重新加载位流后显示按 1-bit 片距 0x3000 取片, 旁听按 0x9000 片首只认 1/3 → 每圈 48 触发卡死。主线同有此隐患 (默认开机靠别的程序先写对)。修: pl_setup 先写 sub01; 仿真 +NOBPP3 复现与板上一致; 位流不变。离线 12/12, 排在 D22 后上板</t>
         </is>
       </c>
       <c r="E148" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fdb4de6</t>
+          <t>dr1v90 task/d21-nband 084bba3</t>
         </is>
       </c>
     </row>
@@ -12188,24 +12188,24 @@
       <c r="A149" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B149" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B149" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
+          <t>上行出口全量复验 45/0, 合主线</t>
         </is>
       </c>
       <c r="E149" s="7" t="inlineStr">
         <is>
-          <t>scratchpad/v_pls4_board.log</t>
+          <t>dr1v90 fdb4de6</t>
         </is>
       </c>
     </row>
@@ -12213,24 +12213,24 @@
       <c r="A150" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B150" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B150" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
+          <t>PL 切片上板: 与 CPU 逐字节一致、30 min 无停摆, 但内容帧率 4.2&lt;15, 退回</t>
         </is>
       </c>
       <c r="E150" s="7" t="inlineStr">
         <is>
-          <t>project_ddr_budget_by_phase_1013</t>
+          <t>scratchpad/v_pls4_board.log</t>
         </is>
       </c>
     </row>
@@ -12250,7 +12250,7 @@
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
+          <t>30 Hz 带载迟到+掉片 3.7% (空载 0.2% 来自旧 netguard), 归因测试中</t>
         </is>
       </c>
       <c r="E151" s="7" t="inlineStr">
@@ -12263,24 +12263,24 @@
       <c r="A152" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B152" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B152" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
+          <t>纯切片带载约 21 min 停摆; 无负载浸泡 2×30 min 不停摆</t>
         </is>
       </c>
       <c r="E152" s="7" t="inlineStr">
         <is>
-          <t>project_short_term_delivery_1013</t>
+          <t>project_ddr_budget_by_phase_1013</t>
         </is>
       </c>
     </row>
@@ -12288,24 +12288,24 @@
       <c r="A153" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B153" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B153" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
         <is>
-          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
+          <t>用户定目标: 复位到亮起 ≤12 s, 找板 ≤20 s</t>
         </is>
       </c>
       <c r="E153" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 debd3cd</t>
+          <t>project_short_term_delivery_1013</t>
         </is>
       </c>
     </row>
@@ -12313,9 +12313,9 @@
       <c r="A154" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B154" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B154" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C154" s="7" t="inlineStr">
@@ -12325,12 +12325,12 @@
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
+          <t>找到 PL 切片器带载停摆根因: 零列描述符丢失 (公共核, 2260 也有) + pop 握手串片, 已修</t>
         </is>
       </c>
       <c r="E154" s="7" t="inlineStr">
         <is>
-          <t>scratchpad v_pls6_board.log</t>
+          <t>dr1v90 task/pls-2047 debd3cd</t>
         </is>
       </c>
     </row>
@@ -12338,9 +12338,9 @@
       <c r="A155" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B155" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B155" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C155" s="7" t="inlineStr">
@@ -12350,12 +12350,12 @@
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
+          <t>上板 60 min 带载 0 停摆、逐字节一致、late 0; 帧率 13.8 差 0.5 退回</t>
         </is>
       </c>
       <c r="E155" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>scratchpad v_pls6_board.log</t>
         </is>
       </c>
     </row>
@@ -12363,24 +12363,24 @@
       <c r="A156" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B156" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B156" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
+          <t>2047 PL 实时切片上板全过: 60 min 带载 0 停摆, 帧率 15.0, 与 CPU 逐字节一致</t>
         </is>
       </c>
       <c r="E156" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d16-ddr 539d303</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -12388,24 +12388,24 @@
       <c r="A157" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B157" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B157" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
+          <t>DDR 慢读根因: 每圈约 1/3 角度每取一列都换行, 两类 CPU 负载叠加越阈值 (0.002%→3%); 建议网格 4×4 分块</t>
         </is>
       </c>
       <c r="E157" s="7" t="inlineStr">
         <is>
-          <t>feedback_save_weekly_quota</t>
+          <t>dr1v90 task/d16-ddr 539d303</t>
         </is>
       </c>
     </row>
@@ -12413,24 +12413,24 @@
       <c r="A158" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B158" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B158" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>V0</t>
+          <t>—</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
+          <t>用户定: 子 agent 并行 ≤5 (周额度); 跑完的 agent 关掉</t>
         </is>
       </c>
       <c r="E158" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/pls-2047 782e9e3</t>
+          <t>feedback_save_weekly_quota</t>
         </is>
       </c>
     </row>
@@ -12438,24 +12438,24 @@
       <c r="A159" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B159" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B159" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>V0</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
+          <t>V0 出口清单: PL 切片上板通过 (D2) 可打勾</t>
         </is>
       </c>
       <c r="E159" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 2364e5c</t>
+          <t>dr1v90 task/pls-2047 782e9e3</t>
         </is>
       </c>
     </row>
@@ -12463,9 +12463,9 @@
       <c r="A160" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B160" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B160" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C160" s="7" t="inlineStr">
@@ -12475,12 +12475,12 @@
       </c>
       <c r="D160" s="7" t="inlineStr">
         <is>
-          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
+          <t>2047 PL 实时切片合进主线 (含公共核两处 bug 修复); D3 上行档位流需按新核重综合</t>
         </is>
       </c>
       <c r="E160" s="7" t="inlineStr">
         <is>
-          <t>用户在场实转</t>
+          <t>dr1v90 2364e5c</t>
         </is>
       </c>
     </row>
@@ -12488,24 +12488,24 @@
       <c r="A161" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B161" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B161" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
-          <t>D18</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D161" s="7" t="inlineStr">
         <is>
-          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
+          <t>PL 硬件切片首次实转上屏 (650 rpm, 完成率 100%, CPU 82% 空闲), 用户确认与 CPU 切片无区别</t>
         </is>
       </c>
       <c r="E161" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>用户在场实转</t>
         </is>
       </c>
     </row>
@@ -12513,9 +12513,9 @@
       <c r="A162" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B162" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B162" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C162" s="7" t="inlineStr">
@@ -12525,12 +12525,12 @@
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
+          <t>用户定: 只保留 PL 切片, 固化开机流程, CPU 切片只留应急退路</t>
         </is>
       </c>
       <c r="E162" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d18-pl-default d35c6d4</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12538,24 +12538,24 @@
       <c r="A163" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B163" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B163" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D18</t>
         </is>
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
-          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
+          <t>开机默认 PL 切片合主线: 上电基础显示 → 推流显示推流 → 停推 5 min 回基础演示; CPU 只留应急退路</t>
         </is>
       </c>
       <c r="E163" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 task/d18-pl-default d35c6d4</t>
         </is>
       </c>
     </row>
@@ -12563,24 +12563,24 @@
       <c r="A164" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B164" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B164" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
+          <t>用户定目标放宽: 亮起 ≤12.5 s / 找板 ≤21 s; V0 出口 ④ 达成</t>
         </is>
       </c>
       <c r="E164" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 dee9be6</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
@@ -12588,24 +12588,24 @@
       <c r="A165" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B165" s="6" t="inlineStr">
-        <is>
-          <t>根因</t>
+      <c r="B165" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>D15b</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
+          <t>无串口远程运维合主线: 升级坏包 (含断网包) 自动回滚后板子能按名字找回; 网络守护不再造成切片迟到 (旧版每分钟 2061 次 → 0); V0 出口 ⑤ 达成</t>
         </is>
       </c>
       <c r="E165" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d15b-color-p2</t>
+          <t>dr1v90 dee9be6</t>
         </is>
       </c>
     </row>
@@ -12613,24 +12613,24 @@
       <c r="A166" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B166" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+      <c r="B166" s="6" t="inlineStr">
+        <is>
+          <t>根因</t>
         </is>
       </c>
       <c r="C166" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D15b</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
+          <t>32 bit PL 全黑: 板端写 LUT 基址仍用 16 bit 布局偏移, PL 把网格当角度表读; 已修 308d1bb, 待上板</t>
         </is>
       </c>
       <c r="E166" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 3a41eb7</t>
+          <t>dr1v90 task/d15b-color-p2</t>
         </is>
       </c>
     </row>
@@ -12638,24 +12638,24 @@
       <c r="A167" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B167" s="6" t="inlineStr">
-        <is>
-          <t>开始</t>
+      <c r="B167" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C167" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
+          <t>WiFi 端 12-bit 通路合主线: 32 bit 像素 PL/CPU 与 CPU 逐字节一致, 2047 上跑通; V0 出口 ⑦ 达成 (7/8)。已知限制: 32 bit 只到 10.83 rps (16.15 rps 时完成率 82-91%)</t>
         </is>
       </c>
       <c r="E167" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 26e69ec soak8h</t>
+          <t>dr1v90 3a41eb7</t>
         </is>
       </c>
     </row>
@@ -12663,24 +12663,24 @@
       <c r="A168" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B168" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B168" s="6" t="inlineStr">
+        <is>
+          <t>开始</t>
         </is>
       </c>
       <c r="C168" s="7" t="inlineStr">
         <is>
-          <t>D16</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
+          <t>8 h 无人值守长跑开跑 19:20 (假转黑屏, 主线 voxslice 0.6 + 卡上 PL 默认; 推 40 min/停 7 min 循环; 判据 S1-S9; 15 min 试跑 9/9)</t>
         </is>
       </c>
       <c r="E168" s="7" t="inlineStr">
         <is>
-          <t>用户 10-14</t>
+          <t>dr1v90 26e69ec soak8h</t>
         </is>
       </c>
     </row>
@@ -12688,49 +12688,49 @@
       <c r="A169" s="17" t="n">
         <v>46309</v>
       </c>
-      <c r="B169" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B169" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C169" s="7" t="inlineStr">
         <is>
-          <t>KR7.2</t>
+          <t>D16</t>
         </is>
       </c>
       <c r="D169" s="7" t="inlineStr">
         <is>
-          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
+          <t>用户批准 QoS 寄存器写入 + 网格 4×4 分块 (D16b 开做, 离线); 长跑后在 2047 做对照</t>
         </is>
       </c>
       <c r="E169" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 5cbe79f</t>
+          <t>用户 10-14</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="17" t="n">
-        <v>46308</v>
-      </c>
-      <c r="B170" s="11" t="inlineStr">
-        <is>
-          <t>交付完成</t>
+        <v>46309</v>
+      </c>
+      <c r="B170" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C170" s="7" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>KR7.2</t>
         </is>
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
+          <t>长跑第 6 段企业 WiFi 踢线 ~5 s, 推流端 voxlive 不重连直接退出 (板端处理正确); 修: voxlive 断线自动重连 5cbe79f; 23:45 重开 8 h</t>
         </is>
       </c>
       <c r="E170" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 b0f6b5d</t>
+          <t>dr1v90 5cbe79f</t>
         </is>
       </c>
     </row>
@@ -12745,17 +12745,17 @@
       </c>
       <c r="C171" s="7" t="inlineStr">
         <is>
-          <t>E7</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="D171" s="7" t="inlineStr">
         <is>
-          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
+          <t>按名字找板 (mDNS) 完成：无串口自重启后 34 s 按名字找到并 ssh 上</t>
         </is>
       </c>
       <c r="E171" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 71d006f / 473abcf</t>
+          <t>dr1v90 b0f6b5d</t>
         </is>
       </c>
     </row>
@@ -12770,17 +12770,17 @@
       </c>
       <c r="C172" s="7" t="inlineStr">
         <is>
-          <t>D1</t>
+          <t>E7</t>
         </is>
       </c>
       <c r="D172" s="7" t="inlineStr">
         <is>
-          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
+          <t>纯切片 30 Hz 位流第一次上硅 D'0–D'3，尾部 late 0.2%，暂停 netguard 后 late/miss 为 0</t>
         </is>
       </c>
       <c r="E172" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 596b191</t>
+          <t>dr1v90 71d006f / 473abcf</t>
         </is>
       </c>
     </row>
@@ -12788,9 +12788,9 @@
       <c r="A173" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B173" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B173" s="11" t="inlineStr">
+        <is>
+          <t>交付完成</t>
         </is>
       </c>
       <c r="C173" s="7" t="inlineStr">
@@ -12800,12 +12800,12 @@
       </c>
       <c r="D173" s="7" t="inlineStr">
         <is>
-          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
+          <t>主机实时推流完成：10 分钟 15.0 fps，NAK 0 / forced 0</t>
         </is>
       </c>
       <c r="E173" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 60c619a / 596b191</t>
+          <t>dr1v90 596b191</t>
         </is>
       </c>
     </row>
@@ -12813,9 +12813,9 @@
       <c r="A174" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B174" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B174" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C174" s="7" t="inlineStr">
@@ -12825,12 +12825,12 @@
       </c>
       <c r="D174" s="7" t="inlineStr">
         <is>
-          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
+          <t>第一次上板端到端延迟 p50 114 ms 未过（停等发送），改发送流水线后降到 84.7 ms</t>
         </is>
       </c>
       <c r="E174" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 9bf16ad</t>
+          <t>dr1v90 60c619a / 596b191</t>
         </is>
       </c>
     </row>
@@ -12838,24 +12838,24 @@
       <c r="A175" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B175" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B175" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C175" s="7" t="inlineStr">
         <is>
-          <t>D4</t>
+          <t>D1</t>
         </is>
       </c>
       <c r="D175" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
+          <t>主会话新克隆独立复验离线+上板全过，合主线（延迟 p50 95 ms / p99 236.6 ms）</t>
         </is>
       </c>
       <c r="E175" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 9bf16ad</t>
         </is>
       </c>
     </row>
@@ -12863,9 +12863,9 @@
       <c r="A176" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B176" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B176" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C176" s="7" t="inlineStr">
@@ -12875,12 +12875,12 @@
       </c>
       <c r="D176" s="7" t="inlineStr">
         <is>
-          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
+          <t>桥接收核对 12-bit 第一次复验 FAIL（新克隆无可执行位），退回</t>
         </is>
       </c>
       <c r="E176" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 6a373d3</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12895,17 +12895,17 @@
       </c>
       <c r="C177" s="7" t="inlineStr">
         <is>
-          <t>D5</t>
+          <t>D4</t>
         </is>
       </c>
       <c r="D177" s="7" t="inlineStr">
         <is>
-          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
+          <t>桥接收核对 12-bit 复验 PASS，合主线</t>
         </is>
       </c>
       <c r="E177" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 cdf49c6</t>
+          <t>dr1v90 6a373d3</t>
         </is>
       </c>
     </row>
@@ -12913,9 +12913,9 @@
       <c r="A178" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B178" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B178" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C178" s="7" t="inlineStr">
@@ -12925,12 +12925,12 @@
       </c>
       <c r="D178" s="7" t="inlineStr">
         <is>
-          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
+          <t>桥驱动 2260 1 期 6 链 24 Hz 12-bit 复验 ALL PASS，合主线</t>
         </is>
       </c>
       <c r="E178" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 cdf49c6</t>
         </is>
       </c>
     </row>
@@ -12950,7 +12950,7 @@
       </c>
       <c r="D179" s="7" t="inlineStr">
         <is>
-          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
+          <t>6 链 4296 片/s 能跑但余量仅 0.40%，瓶颈是桥→2260 链路；留 10% 需 ≤3921 片/s，待用户定</t>
         </is>
       </c>
       <c r="E179" s="7" t="inlineStr">
@@ -12963,24 +12963,24 @@
       <c r="A180" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B180" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B180" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C180" s="7" t="inlineStr">
         <is>
-          <t>D6</t>
+          <t>D5</t>
         </is>
       </c>
       <c r="D180" s="7" t="inlineStr">
         <is>
-          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
+          <t>发现 10-10 验证板 profile 寄存器在 166.67 MHz 下超规格（GCLK 667&gt;600），1 期表已改</t>
         </is>
       </c>
       <c r="E180" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 44ed2cd</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -12988,24 +12988,24 @@
       <c r="A181" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B181" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B181" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C181" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>D6</t>
         </is>
       </c>
       <c r="D181" s="7" t="inlineStr">
         <is>
-          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
+          <t>几何 LUT 生成器逐字节复现 2047 s3lut，verify 22 PASS，合主线</t>
         </is>
       </c>
       <c r="E181" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 44ed2cd</t>
         </is>
       </c>
     </row>
@@ -13013,24 +13013,24 @@
       <c r="A182" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B182" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B182" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C182" s="7" t="inlineStr">
         <is>
-          <t>D14</t>
+          <t>D7</t>
         </is>
       </c>
       <c r="D182" s="7" t="inlineStr">
         <is>
-          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
+          <t>转子运维首次复验 T5 偶发 FAIL，退回返工</t>
         </is>
       </c>
       <c r="E182" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 ffbfeeb</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13045,17 +13045,17 @@
       </c>
       <c r="C183" s="7" t="inlineStr">
         <is>
-          <t>D2</t>
+          <t>D14</t>
         </is>
       </c>
       <c r="D183" s="7" t="inlineStr">
         <is>
-          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
+          <t>10 类内容 + 手机网页遥控离线复验 ALL PASS，用户实转看过（尚未正式上板验收）</t>
         </is>
       </c>
       <c r="E183" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 ffbfeeb</t>
         </is>
       </c>
     </row>
@@ -13063,19 +13063,19 @@
       <c r="A184" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B184" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B184" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C184" s="7" t="inlineStr">
         <is>
-          <t>D12</t>
+          <t>D2</t>
         </is>
       </c>
       <c r="D184" s="7" t="inlineStr">
         <is>
-          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
+          <t>2047 PL 切片离线复验 26/0，待上板（之后 9ba9af0 测试用例过时 26/27 待修）</t>
         </is>
       </c>
       <c r="E184" s="7" t="inlineStr">
@@ -13088,9 +13088,9 @@
       <c r="A185" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B185" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B185" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C185" s="7" t="inlineStr">
@@ -13100,12 +13100,12 @@
       </c>
       <c r="D185" s="7" t="inlineStr">
         <is>
-          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
+          <t>延迟降低上板复验 FAIL：B1 翻页 14.39&lt;15 fps，p99 225 ms，退回</t>
         </is>
       </c>
       <c r="E185" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 764f81d</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13113,24 +13113,24 @@
       <c r="A186" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B186" s="13" t="inlineStr">
-        <is>
-          <t>复验退回</t>
+      <c r="B186" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C186" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12</t>
         </is>
       </c>
       <c r="D186" s="7" t="inlineStr">
         <is>
-          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
+          <t>第二次上板仍未过，根因晚间 WiFi 尾巴（p99 334 vs 白天 48 ms）；判据改为调度问题 0 + 网络晚到 ≤1%，明早主机空闲复测</t>
         </is>
       </c>
       <c r="E186" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 764f81d</t>
         </is>
       </c>
     </row>
@@ -13138,9 +13138,9 @@
       <c r="A187" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B187" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B187" s="13" t="inlineStr">
+        <is>
+          <t>复验退回</t>
         </is>
       </c>
       <c r="C187" s="7" t="inlineStr">
@@ -13150,12 +13150,12 @@
       </c>
       <c r="D187" s="7" t="inlineStr">
         <is>
-          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
+          <t>启动提速上板 FAIL 11 项，但改进已装板保留（6 次重启正常），退回继续压启动时间</t>
         </is>
       </c>
       <c r="E187" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 task/d13-boot fdbb217</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13163,9 +13163,9 @@
       <c r="A188" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B188" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B188" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C188" s="7" t="inlineStr">
@@ -13175,12 +13175,12 @@
       </c>
       <c r="D188" s="7" t="inlineStr">
         <is>
-          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
+          <t>启动提速两轮后：复位→0° 片亮起 38.7→20.1→15.8 s，找板 34→30→25.6 s</t>
         </is>
       </c>
       <c r="E188" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 task/d13-boot fdbb217</t>
         </is>
       </c>
     </row>
@@ -13188,24 +13188,24 @@
       <c r="A189" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B189" s="11" t="inlineStr">
-        <is>
-          <t>复验通过</t>
+      <c r="B189" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
         </is>
       </c>
       <c r="C189" s="7" t="inlineStr">
         <is>
-          <t>D15</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D189" s="7" t="inlineStr">
         <is>
-          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
+          <t>第二步（bootdelay 0 / 精简 uInitrd）写启动文件被权限系统拒绝，需用户明早本人批准后执行</t>
         </is>
       </c>
       <c r="E189" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 1995be8</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13213,24 +13213,24 @@
       <c r="A190" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B190" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B190" s="11" t="inlineStr">
+        <is>
+          <t>复验通过</t>
         </is>
       </c>
       <c r="C190" s="7" t="inlineStr">
         <is>
-          <t>D3;D4;D5</t>
+          <t>D15</t>
         </is>
       </c>
       <c r="D190" s="7" t="inlineStr">
         <is>
-          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
+          <t>WiFi 端 32 bit 像素（X2R10G10B10）阶段 1 复验：黄金/PL 仿真一致，合主线</t>
         </is>
       </c>
       <c r="E190" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 1995be8</t>
         </is>
       </c>
     </row>
@@ -13243,15 +13243,19 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C191" s="7" t="inlineStr"/>
+      <c r="C191" s="7" t="inlineStr">
+        <is>
+          <t>D3;D4;D5</t>
+        </is>
+      </c>
       <c r="D191" s="7" t="inlineStr">
         <is>
-          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
+          <t>下午用户：2260 相关先暂停、先做共用部分（token 不够）；15:00 又改为多开并行恢复 2260</t>
         </is>
       </c>
       <c r="E191" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_sw_three_phases_1013.md</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13259,15 +13263,15 @@
       <c r="A192" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B192" s="19" t="inlineStr">
-        <is>
-          <t>里程碑</t>
+      <c r="B192" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C192" s="7" t="inlineStr"/>
       <c r="D192" s="7" t="inlineStr">
         <is>
-          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
+          <t>软件三期：0 期 2047 屏（现在）/ 1 期 2260 验证板 160×180（预计 11-10 回板）/ 2 期 192×216 目标板；1 期目标 24 Hz / 358 片 / 6 链</t>
         </is>
       </c>
       <c r="E192" s="7" t="inlineStr">
@@ -13280,20 +13284,20 @@
       <c r="A193" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B193" s="18" t="inlineStr">
-        <is>
-          <t>决定</t>
+      <c r="B193" s="19" t="inlineStr">
+        <is>
+          <t>里程碑</t>
         </is>
       </c>
       <c r="C193" s="7" t="inlineStr"/>
       <c r="D193" s="7" t="inlineStr">
         <is>
-          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
+          <t>硬件 1 期验证板预计 2026-11-10 回板（初步交期，可能变），回板前软件能做的都前置</t>
         </is>
       </c>
       <c r="E193" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_arch_common_front_display_backend.md</t>
+          <t>claude_memory/project_sw_three_phases_1013.md</t>
         </is>
       </c>
     </row>
@@ -13306,19 +13310,15 @@
           <t>决定</t>
         </is>
       </c>
-      <c r="C194" s="7" t="inlineStr">
-        <is>
-          <t>D3</t>
-        </is>
-      </c>
+      <c r="C194" s="7" t="inlineStr"/>
       <c r="D194" s="7" t="inlineStr">
         <is>
-          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
+          <t>架构切分：PL 切片器及之前为各期共用的公共部分，屏幕显示为可替换后端，两者之间用实时按角度片流接口</t>
         </is>
       </c>
       <c r="E194" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>claude_memory/project_arch_common_front_display_backend.md</t>
         </is>
       </c>
     </row>
@@ -13333,12 +13333,12 @@
       </c>
       <c r="C195" s="7" t="inlineStr">
         <is>
-          <t>D11</t>
+          <t>D3</t>
         </is>
       </c>
       <c r="D195" s="7" t="inlineStr">
         <is>
-          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
+          <t>用户定：2 期上行 1.2G；1 期保持 24 Hz（358 片，桥链路余量 0.40%）不降档</t>
         </is>
       </c>
       <c r="E195" s="7" t="inlineStr">
@@ -13358,12 +13358,12 @@
       </c>
       <c r="C196" s="7" t="inlineStr">
         <is>
-          <t>D12;D13;D14</t>
+          <t>D11</t>
         </is>
       </c>
       <c r="D196" s="7" t="inlineStr">
         <is>
-          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
+          <t>傍晚用户：杜邦线跑不了 1.2G，1.2G 实测等 V1 回板；C1 台架只做 ≤300M 低速功能档</t>
         </is>
       </c>
       <c r="E196" s="7" t="inlineStr">
@@ -13383,12 +13383,12 @@
       </c>
       <c r="C197" s="7" t="inlineStr">
         <is>
-          <t>D13</t>
+          <t>D12;D13;D14</t>
         </is>
       </c>
       <c r="D197" s="7" t="inlineStr">
         <is>
-          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
+          <t>19:00 用户：V0 可见的先插队、V1 接着做，新派 D12 延迟降低 / D13 启动提速 / D14 内容与手机控制</t>
         </is>
       </c>
       <c r="E197" s="7" t="inlineStr">
@@ -13408,12 +13408,12 @@
       </c>
       <c r="C198" s="7" t="inlineStr">
         <is>
-          <t>D15;D16</t>
+          <t>D13</t>
         </is>
       </c>
       <c r="D198" s="7" t="inlineStr">
         <is>
-          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
+          <t>21:10 用户定 D13 目标：复位到 0° 片亮起 ≤12 s，找板 ≤20 s（看板 KR8.1 已改）</t>
         </is>
       </c>
       <c r="E198" s="7" t="inlineStr">
@@ -13433,17 +13433,17 @@
       </c>
       <c r="C199" s="7" t="inlineStr">
         <is>
-          <t>KR5.2</t>
+          <t>D15;D16</t>
         </is>
       </c>
       <c r="D199" s="7" t="inlineStr">
         <is>
-          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
+          <t>用户选 12-bit 方案 A：WiFi 端传高位宽、像素位宽 16/32 bit 可配（D15）；DDR 做到极限 A 线（D16），B 线并入 T2 硬件</t>
         </is>
       </c>
       <c r="E199" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 49031f6</t>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
         </is>
       </c>
     </row>
@@ -13451,24 +13451,24 @@
       <c r="A200" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B200" s="15" t="inlineStr">
-        <is>
-          <t>问题</t>
+      <c r="B200" s="18" t="inlineStr">
+        <is>
+          <t>决定</t>
         </is>
       </c>
       <c r="C200" s="7" t="inlineStr">
         <is>
-          <t>D7</t>
+          <t>KR5.2</t>
         </is>
       </c>
       <c r="D200" s="7" t="inlineStr">
         <is>
-          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+          <t>用户实转核实：2047 旧表镜像，已更正为新表 0decad54</t>
         </is>
       </c>
       <c r="E200" s="7" t="inlineStr">
         <is>
-          <t>claude_memory/project_short_term_delivery_1013.md</t>
+          <t>dr1v90 49031f6</t>
         </is>
       </c>
     </row>
@@ -13476,18 +13476,43 @@
       <c r="A201" s="17" t="n">
         <v>46308</v>
       </c>
-      <c r="B201" s="19" t="inlineStr">
+      <c r="B201" s="15" t="inlineStr">
+        <is>
+          <t>问题</t>
+        </is>
+      </c>
+      <c r="C201" s="7" t="inlineStr">
+        <is>
+          <t>D7</t>
+        </is>
+      </c>
+      <c r="D201" s="7" t="inlineStr">
+        <is>
+          <t>D7 上板补测会装/还原 autorun，冲掉 D13 补丁，须排在 D13 定稿合并之后；夜间板子排程 D12→D13→D2→D7→8 h 长跑</t>
+        </is>
+      </c>
+      <c r="E201" s="7" t="inlineStr">
+        <is>
+          <t>claude_memory/project_short_term_delivery_1013.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="17" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B202" s="19" t="inlineStr">
         <is>
           <t>里程碑</t>
         </is>
       </c>
-      <c r="C201" s="7" t="inlineStr"/>
-      <c r="D201" s="7" t="inlineStr">
+      <c r="C202" s="7" t="inlineStr"/>
+      <c r="D202" s="7" t="inlineStr">
         <is>
           <t>显性目的进度看板第一版建立：10 个显性目的 + KR 趋势 + 燃起图 + 里程碑趋势</t>
         </is>
       </c>
-      <c r="E201" s="7" t="inlineStr">
+      <c r="E202" s="7" t="inlineStr">
         <is>
           <t>claude_memory/project_progress_dashboard.md</t>
         </is>
@@ -18355,7 +18380,7 @@
         <v>29</v>
       </c>
       <c r="D11" s="6" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="12">
@@ -19995,15 +20020,17 @@
       <c r="E65" s="17" t="n">
         <v>46315</v>
       </c>
-      <c r="F65" s="17" t="n"/>
-      <c r="G65" s="15" t="inlineStr">
-        <is>
-          <t>🔄</t>
+      <c r="F65" s="17" t="n">
+        <v>46314</v>
+      </c>
+      <c r="G65" s="11" t="inlineStr">
+        <is>
+          <t>✅</t>
         </is>
       </c>
       <c r="H65" s="7" t="inlineStr">
         <is>
-          <t>方案 be3b699 已上 03 (uboot.env); 软重启 20/20 进内核; 冷上电 20 次等 USB 继电器 (LCUS-1) 到货自动跑</t>
+          <t>方案 be3b699 (只改 uboot.env); 03 软重启 20/20 + 手动冷上电 20/20 进内核到 login (0 次停 =&gt;; -110 探测仍刷但 env/boot.scr 正常读); 日志 progress/d29_coldboot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
[看板] KR7.2 记 02 24 h 长跑 PASS (V2 目标 24 h 达标)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/progress/显性目的进度_2026-10-19.xlsx
+++ b/docs/progress/显性目的进度_2026-10-19.xlsx
@@ -15,7 +15,7 @@
     <sheet name="历史记录" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'历史记录'!$A$1:$I$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2749,12 +2749,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'指标趋势'!$A$277:$A$280</f>
+              <f>'指标趋势'!$A$277:$A$281</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'指标趋势'!$B$277:$B$280</f>
+              <f>'指标趋势'!$B$277:$B$281</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -2792,12 +2792,12 @@
           </marker>
           <xVal>
             <numRef>
-              <f>'指标趋势'!$A$277:$A$280</f>
+              <f>'指标趋势'!$A$277:$A$281</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'指标趋势'!$C$277:$C$280</f>
+              <f>'指标趋势'!$C$277:$C$281</f>
             </numRef>
           </yVal>
           <smooth val="0"/>
@@ -2917,7 +2917,7 @@
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
-          <max val="46310"/>
+          <max val="46312"/>
           <min val="46307"/>
         </scaling>
         <delete val="0"/>
@@ -8700,16 +8700,16 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>0.8108108108108109</v>
+        <v>0.8243243243243243</v>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>60/74</t>
+          <t>61/74</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>KR 15/24 + 交付 45/50 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
+          <t>KR 16/24 + 交付 45/50 — 交付的"需要"是嵌套的：V0 需要 = 阶段 V0；V1 需要 = V0 + V1准备；V2 需要 = V1 需要 + V2 (阶段列见 deliverables.csv，没填阶段的交付不计)。</t>
         </is>
       </c>
       <c r="G6" s="8" t="n">
@@ -8827,7 +8827,7 @@
         <v>0.8676</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>0.8108</v>
+        <v>0.8243</v>
       </c>
     </row>
     <row r="12">
@@ -14708,10 +14708,10 @@
         </is>
       </c>
       <c r="I20" s="6" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="J20" s="17" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="K20" s="7" t="inlineStr">
         <is>
@@ -14734,11 +14734,11 @@
       </c>
       <c r="P20" s="7" t="inlineStr">
         <is>
-          <t>dr1v90 fe53bde; progress/soak_v0/report.md</t>
+          <t>progress/soak_v0/1016_wkend_24h</t>
         </is>
       </c>
       <c r="Q20" s="21" t="n">
-        <v>0.3333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="21">
@@ -17311,19 +17311,19 @@
       </c>
       <c r="C278" s="6" t="n"/>
       <c r="D278" s="8" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="E278" s="6" t="n">
         <v>8</v>
       </c>
       <c r="F278" s="8" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="G278" s="6" t="n">
         <v>8</v>
       </c>
       <c r="H278" s="8" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
       <c r="I278" s="6" t="n">
         <v>24</v>
@@ -17346,6 +17346,15 @@
         <v>8</v>
       </c>
       <c r="C280" s="6" t="n"/>
+    </row>
+    <row r="281">
+      <c r="A281" s="8" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B281" s="6" t="n">
+        <v>24</v>
+      </c>
+      <c r="C281" s="6" t="n"/>
     </row>
     <row r="292">
       <c r="A292" s="27" t="inlineStr">
@@ -20620,7 +20629,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I80"/>
+  <dimension ref="A1:I81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -23920,8 +23929,49 @@
         </is>
       </c>
     </row>
+    <row r="81">
+      <c r="A81" s="29" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B81" s="7" t="n">
+        <v>7</v>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>KR7.2</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>连续无故障: 软件链路 (假转, 无人值守)</t>
+        </is>
+      </c>
+      <c r="E81" s="7" t="inlineStr">
+        <is>
+          <t>h</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="n">
+        <v>24</v>
+      </c>
+      <c r="G81" s="7" t="inlineStr">
+        <is>
+          <t>V0 2047</t>
+        </is>
+      </c>
+      <c r="H81" s="7" t="inlineStr">
+        <is>
+          <t>progress/soak_v0/1016_wkend_24h</t>
+        </is>
+      </c>
+      <c r="I81" s="7" t="inlineStr">
+        <is>
+          <t>02 产品配置 24 h 长跑 PASS 10/10 (主线 8eced5a); 03 24 h 9/10 (WiFi 断 155 s, D22b 已修)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:I80"/>
+  <autoFilter ref="A1:I81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>